<commit_message>
feat: upgrade Quarterly Tax System to v2 — adds Dashboard, Examples, 15-page bonus PDF
Spreadsheet (now 9 tabs, 26 KB):
- New Dashboard tab — KPI cards for annual totals, YTD paid, remaining
  balance, safe-harbor status, next deadline countdown, plus a Q1–Q4
  target-vs-paid bar chart
- New Examples tab — 3 fully worked-out scenarios (DoorDash full-timer,
  freelancer + W-2, Etsy seller) with every input and output filled in

Bonus PDF (new, 15 pages, 30 KB):
- The Self-Employed Quarterly Tax Survival Guide 2026
- Cover + 10 chapters: why quarterly taxes exist, penalty math, both
  safe-harbor rules, how to calculate, the four deadlines, state systems,
  where to pay, missed-quarter recovery, common mistakes, quick-ref card

Site funnel:
- All 32 existing quarterly product cards refreshed to advertise the
  bonus PDF + new tabs. Price unchanged at $17, but the value
  proposition now actually matches the price.
- Listing copy and inject script updated to match the v2 product.
</commit_message>
<xml_diff>
--- a/products/quarterly-tax-system-2026.xlsx
+++ b/products/quarterly-tax-system-2026.xlsx
@@ -8,12 +8,14 @@
   </bookViews>
   <sheets>
     <sheet name="Start Here" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Setup" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Income Forecast" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Tax Calculator" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Quarterly Payments" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Safe Harbor" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="IRS Reference" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Setup" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Income Forecast" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Tax Calculator" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Quarterly Payments" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Safe Harbor" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Examples" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="IRS Reference" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName name="TaxYear">Setup!$C$6</definedName>
@@ -56,7 +58,7 @@
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0"/>
     <numFmt numFmtId="166" formatCode="yyyy-mm-dd"/>
   </numFmts>
-  <fonts count="14">
+  <fonts count="19">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -140,8 +142,38 @@
       <color rgb="FFC9973A"/>
       <sz val="12"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="FF1C2B4A"/>
+      <sz val="24"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="FFC9973A"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="FF6B7A96"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="FFB83232"/>
+      <sz val="22"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="FF1C2B4A"/>
+      <sz val="16"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -172,8 +204,20 @@
         <bgColor rgb="FFF0ECE3"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFAF8F4"/>
+        <bgColor rgb="FFFAF8F4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFBE9E9"/>
+        <bgColor rgb="FFFBE9E9"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="11">
+  <borders count="18">
     <border>
       <left/>
       <right/>
@@ -300,11 +344,86 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFE5E7ED"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFE5E7ED"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFE5E7ED"/>
+      </top>
+      <bottom/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFE5E7ED"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFE5E7ED"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFE5E7ED"/>
+      </bottom>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFE5E7ED"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFE5E7ED"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFE5E7ED"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFE5E7ED"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFE5E7ED"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFE5E7ED"/>
+      </top>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFE5E7ED"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFE5E7ED"/>
+      </right>
+      <bottom style="thin">
+        <color rgb="FFE5E7ED"/>
+      </bottom>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFE5E7ED"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="59">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -341,15 +460,61 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="6" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="3" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="10" fillId="6" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="5" fillId="3" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="17" fillId="7" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="6" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="18" fillId="6" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
@@ -364,9 +529,6 @@
     </xf>
     <xf numFmtId="164" fontId="4" fillId="3" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -399,6 +561,22 @@
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -407,7 +585,35 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="6">
+  <dxfs count="8">
+    <dxf>
+      <font>
+        <name val="Calibri"/>
+        <b val="1"/>
+        <color rgb="FF276944"/>
+        <sz val="16"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFEAF5EF"/>
+          <bgColor rgb="FFEAF5EF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Calibri"/>
+        <b val="1"/>
+        <color rgb="FFA86C0A"/>
+        <sz val="16"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFEF6E8"/>
+          <bgColor rgb="FFFEF6E8"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <b val="1"/>
@@ -554,6 +760,179 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="11"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Federal — Target vs Paid by Quarter</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Dashboard'!C22</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill>
+              <a:srgbClr val="1C2B4A"/>
+            </a:solidFill>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Dashboard'!$B$23:$B$26</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Dashboard'!$C$23:$C$26</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'Dashboard'!D22</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill>
+              <a:srgbClr val="C9973A"/>
+            </a:solidFill>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Dashboard'!$B$23:$B$26</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Dashboard'!$D$23:$D$26</f>
+            </numRef>
+          </val>
+        </ser>
+        <dLbls>
+          <showVal val="0"/>
+        </dLbls>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Quarter</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Dollars</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>21</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6480000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1130,6 +1509,329 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="B2:J40"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="2" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="2" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="2" ht="36" customHeight="1">
+      <c r="B2" s="14" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" s="15" t="inlineStr">
+        <is>
+          <t>One screen — where you stand right now. All values update as you fill in the other tabs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="24" customHeight="1">
+      <c r="B5" s="16" t="inlineStr">
+        <is>
+          <t>ANNUAL TAX PICTURE</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="24" customHeight="1">
+      <c r="B6" s="17" t="inlineStr">
+        <is>
+          <t>TOTAL SE TAX</t>
+        </is>
+      </c>
+      <c r="C6" s="18" t="n"/>
+      <c r="D6" s="17" t="inlineStr">
+        <is>
+          <t>FEDERAL INCOME TAX</t>
+        </is>
+      </c>
+      <c r="E6" s="18" t="n"/>
+      <c r="G6" s="17" t="inlineStr">
+        <is>
+          <t>STATE TAX</t>
+        </is>
+      </c>
+      <c r="H6" s="18" t="n"/>
+      <c r="I6" s="19" t="inlineStr">
+        <is>
+          <t>TOTAL ANNUAL OWED</t>
+        </is>
+      </c>
+      <c r="J6" s="18" t="n"/>
+    </row>
+    <row r="7" ht="40" customHeight="1">
+      <c r="B7" s="20">
+        <f>SETax</f>
+        <v/>
+      </c>
+      <c r="C7" s="21" t="n"/>
+      <c r="D7" s="20">
+        <f>FedIncomeTax</f>
+        <v/>
+      </c>
+      <c r="E7" s="21" t="n"/>
+      <c r="G7" s="20">
+        <f>'Tax Calculator'!$C$20</f>
+        <v/>
+      </c>
+      <c r="H7" s="21" t="n"/>
+      <c r="I7" s="22">
+        <f>SETax+FedIncomeTax+'Tax Calculator'!$C$20</f>
+        <v/>
+      </c>
+      <c r="J7" s="21" t="n"/>
+    </row>
+    <row r="9" ht="12" customHeight="1"/>
+    <row r="10" ht="24" customHeight="1">
+      <c r="B10" s="16" t="inlineStr">
+        <is>
+          <t>WHERE YOU STAND TODAY</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="24" customHeight="1">
+      <c r="B11" s="17" t="inlineStr">
+        <is>
+          <t>FED PAID YTD</t>
+        </is>
+      </c>
+      <c r="C11" s="18" t="n"/>
+      <c r="D11" s="17" t="inlineStr">
+        <is>
+          <t>STATE PAID YTD</t>
+        </is>
+      </c>
+      <c r="E11" s="18" t="n"/>
+      <c r="G11" s="17" t="inlineStr">
+        <is>
+          <t>FEDERAL TARGET (annual)</t>
+        </is>
+      </c>
+      <c r="H11" s="18" t="n"/>
+      <c r="I11" s="23" t="inlineStr">
+        <is>
+          <t>REMAINING FEDERAL</t>
+        </is>
+      </c>
+      <c r="J11" s="18" t="n"/>
+    </row>
+    <row r="12" ht="40" customHeight="1">
+      <c r="B12" s="20">
+        <f>FedPaidYTD</f>
+        <v/>
+      </c>
+      <c r="C12" s="21" t="n"/>
+      <c r="D12" s="20">
+        <f>StatePaidYTD</f>
+        <v/>
+      </c>
+      <c r="E12" s="21" t="n"/>
+      <c r="G12" s="20">
+        <f>NetFedOwed</f>
+        <v/>
+      </c>
+      <c r="H12" s="21" t="n"/>
+      <c r="I12" s="24">
+        <f>MAX(NetFedOwed-FedPaidYTD,0)</f>
+        <v/>
+      </c>
+      <c r="J12" s="21" t="n"/>
+    </row>
+    <row r="14" ht="12" customHeight="1"/>
+    <row r="15" ht="24" customHeight="1">
+      <c r="B15" s="16" t="inlineStr">
+        <is>
+          <t>SAFETY &amp; NEXT DEADLINE</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="24" customHeight="1">
+      <c r="B16" s="25" t="inlineStr">
+        <is>
+          <t>PENALTY-SAFE STATUS</t>
+        </is>
+      </c>
+      <c r="C16" s="26" t="n"/>
+      <c r="D16" s="26" t="n"/>
+      <c r="E16" s="18" t="n"/>
+      <c r="G16" s="25" t="inlineStr">
+        <is>
+          <t>NEXT QUARTERLY DEADLINE</t>
+        </is>
+      </c>
+      <c r="H16" s="26" t="n"/>
+      <c r="I16" s="26" t="n"/>
+      <c r="J16" s="18" t="n"/>
+    </row>
+    <row r="17" ht="44" customHeight="1">
+      <c r="B17" s="27">
+        <f>IF(OR('Safe Harbor'!$C$8&gt;='Safe Harbor'!$C$7,'Safe Harbor'!$C$14&gt;='Safe Harbor'!$C$13),"✓ Penalty-safe","⚠ Not yet penalty-safe")</f>
+        <v/>
+      </c>
+      <c r="C17" s="28" t="n"/>
+      <c r="D17" s="28" t="n"/>
+      <c r="E17" s="21" t="n"/>
+      <c r="G17" s="29">
+        <f>IF(TODAY()&lt;=DATE(TaxYear,4,15),"Q1 — April 15, "&amp;TEXT(DATE(TaxYear,4,15)-TODAY(),"0")&amp;" days away",IF(TODAY()&lt;=DATE(TaxYear,6,15),"Q2 — June 15, "&amp;TEXT(DATE(TaxYear,6,15)-TODAY(),"0")&amp;" days away",IF(TODAY()&lt;=DATE(TaxYear,9,15),"Q3 — September 15, "&amp;TEXT(DATE(TaxYear,9,15)-TODAY(),"0")&amp;" days away",IF(TODAY()&lt;=DATE(TaxYear+1,1,15),"Q4 — January 15 (next year), "&amp;TEXT(DATE(TaxYear+1,1,15)-TODAY(),"0")&amp;" days away","All quarterly deadlines passed for "&amp;TaxYear))))</f>
+        <v/>
+      </c>
+      <c r="H17" s="28" t="n"/>
+      <c r="I17" s="28" t="n"/>
+      <c r="J17" s="21" t="n"/>
+    </row>
+    <row r="19" ht="12" customHeight="1"/>
+    <row r="20" ht="24" customHeight="1">
+      <c r="B20" s="16" t="inlineStr">
+        <is>
+          <t>QUARTERLY PROGRESS — FEDERAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="18" customHeight="1">
+      <c r="B22" s="30" t="inlineStr">
+        <is>
+          <t>Quarter</t>
+        </is>
+      </c>
+      <c r="C22" s="31" t="inlineStr">
+        <is>
+          <t>Target $</t>
+        </is>
+      </c>
+      <c r="D22" s="31" t="inlineStr">
+        <is>
+          <t>Paid $</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="18" customHeight="1">
+      <c r="B23" s="30" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="C23" s="32">
+        <f>'Quarterly Payments'!$D$7</f>
+        <v/>
+      </c>
+      <c r="D23" s="32">
+        <f>'Quarterly Payments'!$F$7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24" ht="18" customHeight="1">
+      <c r="B24" s="30" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
+      <c r="C24" s="32">
+        <f>'Quarterly Payments'!$D$8</f>
+        <v/>
+      </c>
+      <c r="D24" s="32">
+        <f>'Quarterly Payments'!$F$8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25" ht="18" customHeight="1">
+      <c r="B25" s="30" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="C25" s="32">
+        <f>'Quarterly Payments'!$D$9</f>
+        <v/>
+      </c>
+      <c r="D25" s="32">
+        <f>'Quarterly Payments'!$F$9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26" ht="18" customHeight="1">
+      <c r="B26" s="30" t="inlineStr">
+        <is>
+          <t>Q4</t>
+        </is>
+      </c>
+      <c r="C26" s="32">
+        <f>'Quarterly Payments'!$D$10</f>
+        <v/>
+      </c>
+      <c r="D26" s="32">
+        <f>'Quarterly Payments'!$F$10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40" ht="40" customHeight="1">
+      <c r="B40" s="33" t="inlineStr">
+        <is>
+          <t>Everything on this Dashboard is calculated from the Setup, Income Forecast, and Quarterly Payments tabs. If a number looks wrong, the source is on those tabs — not here.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="27">
+    <mergeCell ref="G12:H12"/>
+    <mergeCell ref="I6:J6"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="G11:H11"/>
+    <mergeCell ref="I11:J11"/>
+    <mergeCell ref="G16:J16"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="G7:H7"/>
+    <mergeCell ref="B10:J10"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="I7:J7"/>
+    <mergeCell ref="D11:E11"/>
+    <mergeCell ref="B16:E16"/>
+    <mergeCell ref="B40:J40"/>
+    <mergeCell ref="G6:H6"/>
+    <mergeCell ref="B15:J15"/>
+    <mergeCell ref="I12:J12"/>
+    <mergeCell ref="B5:J5"/>
+    <mergeCell ref="D7:E7"/>
+    <mergeCell ref="G17:J17"/>
+    <mergeCell ref="B20:J20"/>
+    <mergeCell ref="D12:E12"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="B17:E17"/>
+    <mergeCell ref="B3:J3"/>
+    <mergeCell ref="B2:J2"/>
+  </mergeCells>
+  <conditionalFormatting sqref="B17">
+    <cfRule type="expression" priority="1" dxfId="0">
+      <formula>ISNUMBER(SEARCH("safe",B17))</formula>
+    </cfRule>
+    <cfRule type="expression" priority="2" dxfId="1">
+      <formula>ISNUMBER(SEARCH("Not yet",B17))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="B2:D36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1140,7 +1842,7 @@
   </cols>
   <sheetData>
     <row r="2" ht="32" customHeight="1">
-      <c r="B2" s="14" t="inlineStr">
+      <c r="B2" s="34" t="inlineStr">
         <is>
           <t>Setup</t>
         </is>
@@ -1161,12 +1863,12 @@
       </c>
     </row>
     <row r="6" ht="24" customHeight="1">
-      <c r="B6" s="16" t="inlineStr">
+      <c r="B6" s="30" t="inlineStr">
         <is>
           <t>Tax year</t>
         </is>
       </c>
-      <c r="C6" s="17" t="n">
+      <c r="C6" s="35" t="n">
         <v>2026</v>
       </c>
       <c r="D6" s="15" t="inlineStr">
@@ -1176,12 +1878,12 @@
       </c>
     </row>
     <row r="7" ht="24" customHeight="1">
-      <c r="B7" s="16" t="inlineStr">
+      <c r="B7" s="30" t="inlineStr">
         <is>
           <t>Filing status</t>
         </is>
       </c>
-      <c r="C7" s="17" t="inlineStr">
+      <c r="C7" s="35" t="inlineStr">
         <is>
           <t>Single</t>
         </is>
@@ -1193,12 +1895,12 @@
       </c>
     </row>
     <row r="8" ht="24" customHeight="1">
-      <c r="B8" s="16" t="inlineStr">
+      <c r="B8" s="30" t="inlineStr">
         <is>
           <t>State</t>
         </is>
       </c>
-      <c r="C8" s="17" t="inlineStr">
+      <c r="C8" s="35" t="inlineStr">
         <is>
           <t>CA</t>
         </is>
@@ -1210,12 +1912,12 @@
       </c>
     </row>
     <row r="9" ht="24" customHeight="1">
-      <c r="B9" s="16" t="inlineStr">
+      <c r="B9" s="30" t="inlineStr">
         <is>
           <t>State flat estimated tax rate</t>
         </is>
       </c>
-      <c r="C9" s="18" t="n">
+      <c r="C9" s="36" t="n">
         <v>0.06</v>
       </c>
       <c r="D9" s="15" t="inlineStr">
@@ -1232,12 +1934,12 @@
       </c>
     </row>
     <row r="12" ht="24" customHeight="1">
-      <c r="B12" s="16" t="inlineStr">
+      <c r="B12" s="30" t="inlineStr">
         <is>
           <t>Estimated net self-employment income (annual)</t>
         </is>
       </c>
-      <c r="C12" s="19" t="n">
+      <c r="C12" s="37" t="n">
         <v>0</v>
       </c>
       <c r="D12" s="15" t="inlineStr">
@@ -1247,12 +1949,12 @@
       </c>
     </row>
     <row r="13" ht="24" customHeight="1">
-      <c r="B13" s="16" t="inlineStr">
+      <c r="B13" s="30" t="inlineStr">
         <is>
           <t>W-2 income (if you also have a day job)</t>
         </is>
       </c>
-      <c r="C13" s="19" t="n">
+      <c r="C13" s="37" t="n">
         <v>0</v>
       </c>
       <c r="D13" s="15" t="inlineStr">
@@ -1262,12 +1964,12 @@
       </c>
     </row>
     <row r="14" ht="24" customHeight="1">
-      <c r="B14" s="16" t="inlineStr">
+      <c r="B14" s="30" t="inlineStr">
         <is>
           <t>Federal tax withheld from W-2 (this year)</t>
         </is>
       </c>
-      <c r="C14" s="19" t="n">
+      <c r="C14" s="37" t="n">
         <v>0</v>
       </c>
       <c r="D14" s="15" t="inlineStr">
@@ -1284,12 +1986,12 @@
       </c>
     </row>
     <row r="17" ht="24" customHeight="1">
-      <c r="B17" s="16" t="inlineStr">
+      <c r="B17" s="30" t="inlineStr">
         <is>
           <t>Total federal tax owed last year (Form 1040 line 24)</t>
         </is>
       </c>
-      <c r="C17" s="19" t="n">
+      <c r="C17" s="37" t="n">
         <v>0</v>
       </c>
       <c r="D17" s="15" t="inlineStr">
@@ -1299,12 +2001,12 @@
       </c>
     </row>
     <row r="18" ht="24" customHeight="1">
-      <c r="B18" s="16" t="inlineStr">
+      <c r="B18" s="30" t="inlineStr">
         <is>
           <t>Last year's AGI (Form 1040 line 11)</t>
         </is>
       </c>
-      <c r="C18" s="19" t="n">
+      <c r="C18" s="37" t="n">
         <v>0</v>
       </c>
       <c r="D18" s="15" t="inlineStr">
@@ -1321,12 +2023,12 @@
       </c>
     </row>
     <row r="21" ht="24" customHeight="1">
-      <c r="B21" s="16" t="inlineStr">
+      <c r="B21" s="30" t="inlineStr">
         <is>
           <t>Standard deduction (single / MFS)</t>
         </is>
       </c>
-      <c r="C21" s="19" t="n">
+      <c r="C21" s="37" t="n">
         <v>15750</v>
       </c>
       <c r="D21" s="15" t="inlineStr">
@@ -1336,12 +2038,12 @@
       </c>
     </row>
     <row r="22" ht="24" customHeight="1">
-      <c r="B22" s="16" t="inlineStr">
+      <c r="B22" s="30" t="inlineStr">
         <is>
           <t>Standard deduction (MFJ)</t>
         </is>
       </c>
-      <c r="C22" s="19" t="n">
+      <c r="C22" s="37" t="n">
         <v>31500</v>
       </c>
       <c r="D22" s="15" t="inlineStr">
@@ -1351,12 +2053,12 @@
       </c>
     </row>
     <row r="23" ht="24" customHeight="1">
-      <c r="B23" s="16" t="inlineStr">
+      <c r="B23" s="30" t="inlineStr">
         <is>
           <t>Standard deduction (HOH)</t>
         </is>
       </c>
-      <c r="C23" s="19" t="n">
+      <c r="C23" s="37" t="n">
         <v>23625</v>
       </c>
       <c r="D23" s="15" t="inlineStr">
@@ -1366,12 +2068,12 @@
       </c>
     </row>
     <row r="24" ht="24" customHeight="1">
-      <c r="B24" s="16" t="inlineStr">
+      <c r="B24" s="30" t="inlineStr">
         <is>
           <t>Social Security wage base</t>
         </is>
       </c>
-      <c r="C24" s="19" t="n">
+      <c r="C24" s="37" t="n">
         <v>176100</v>
       </c>
       <c r="D24" s="15" t="inlineStr">
@@ -1405,84 +2107,84 @@
       </c>
     </row>
     <row r="28" ht="20" customHeight="1">
-      <c r="B28" s="20" t="n">
+      <c r="B28" s="38" t="n">
         <v>11925</v>
       </c>
-      <c r="C28" s="20" t="n">
+      <c r="C28" s="38" t="n">
         <v>23850</v>
       </c>
-      <c r="D28" s="21" t="n">
+      <c r="D28" s="39" t="n">
         <v>0.1</v>
       </c>
     </row>
     <row r="29" ht="20" customHeight="1">
-      <c r="B29" s="20" t="n">
+      <c r="B29" s="38" t="n">
         <v>48475</v>
       </c>
-      <c r="C29" s="20" t="n">
+      <c r="C29" s="38" t="n">
         <v>96950</v>
       </c>
-      <c r="D29" s="21" t="n">
+      <c r="D29" s="39" t="n">
         <v>0.12</v>
       </c>
     </row>
     <row r="30" ht="20" customHeight="1">
-      <c r="B30" s="20" t="n">
+      <c r="B30" s="38" t="n">
         <v>103350</v>
       </c>
-      <c r="C30" s="20" t="n">
+      <c r="C30" s="38" t="n">
         <v>206700</v>
       </c>
-      <c r="D30" s="21" t="n">
+      <c r="D30" s="39" t="n">
         <v>0.22</v>
       </c>
     </row>
     <row r="31" ht="20" customHeight="1">
-      <c r="B31" s="20" t="n">
+      <c r="B31" s="38" t="n">
         <v>197300</v>
       </c>
-      <c r="C31" s="20" t="n">
+      <c r="C31" s="38" t="n">
         <v>394600</v>
       </c>
-      <c r="D31" s="21" t="n">
+      <c r="D31" s="39" t="n">
         <v>0.24</v>
       </c>
     </row>
     <row r="32" ht="20" customHeight="1">
-      <c r="B32" s="20" t="n">
+      <c r="B32" s="38" t="n">
         <v>250525</v>
       </c>
-      <c r="C32" s="20" t="n">
+      <c r="C32" s="38" t="n">
         <v>501050</v>
       </c>
-      <c r="D32" s="21" t="n">
+      <c r="D32" s="39" t="n">
         <v>0.32</v>
       </c>
     </row>
     <row r="33" ht="20" customHeight="1">
-      <c r="B33" s="20" t="n">
+      <c r="B33" s="38" t="n">
         <v>626350</v>
       </c>
-      <c r="C33" s="20" t="n">
+      <c r="C33" s="38" t="n">
         <v>751600</v>
       </c>
-      <c r="D33" s="21" t="n">
+      <c r="D33" s="39" t="n">
         <v>0.35</v>
       </c>
     </row>
     <row r="34" ht="20" customHeight="1">
-      <c r="B34" s="20" t="n">
+      <c r="B34" s="38" t="n">
         <v>999999999</v>
       </c>
-      <c r="C34" s="20" t="n">
+      <c r="C34" s="38" t="n">
         <v>999999999</v>
       </c>
-      <c r="D34" s="21" t="n">
+      <c r="D34" s="39" t="n">
         <v>0.37</v>
       </c>
     </row>
     <row r="36" ht="36" customHeight="1">
-      <c r="B36" s="22" t="inlineStr">
+      <c r="B36" s="33" t="inlineStr">
         <is>
           <t>HoH and MFS brackets aren't modeled separately — if you use those statuses, set filing status above to the closest match (HOH → MFJ for brackets, MFS → Single) and adjust the standard deduction. For complex returns, consult a CPA.</t>
         </is>
@@ -1508,7 +2210,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1530,7 +2232,7 @@
   </cols>
   <sheetData>
     <row r="2" ht="32" customHeight="1">
-      <c r="B2" s="14" t="inlineStr">
+      <c r="B2" s="34" t="inlineStr">
         <is>
           <t>Income Forecast</t>
         </is>
@@ -1586,7 +2288,7 @@
           <t>Other</t>
         </is>
       </c>
-      <c r="I5" s="23" t="inlineStr">
+      <c r="I5" s="40" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
@@ -1598,25 +2300,25 @@
           <t>January</t>
         </is>
       </c>
-      <c r="C6" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="D6" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="E6" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="F6" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G6" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H6" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="I6" s="24">
+      <c r="C6" s="38" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" s="38" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" s="38" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" s="38" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" s="38" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" s="38" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" s="41">
         <f>SUM(C6:H6)</f>
         <v/>
       </c>
@@ -1627,25 +2329,25 @@
           <t>February</t>
         </is>
       </c>
-      <c r="C7" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="D7" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="E7" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="F7" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G7" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H7" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="I7" s="24">
+      <c r="C7" s="38" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" s="38" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" s="38" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" s="38" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" s="38" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" s="38" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" s="41">
         <f>SUM(C7:H7)</f>
         <v/>
       </c>
@@ -1656,25 +2358,25 @@
           <t>March</t>
         </is>
       </c>
-      <c r="C8" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="D8" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="E8" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="F8" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G8" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H8" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="I8" s="24">
+      <c r="C8" s="38" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" s="38" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" s="38" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" s="38" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="38" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" s="38" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" s="41">
         <f>SUM(C8:H8)</f>
         <v/>
       </c>
@@ -1685,25 +2387,25 @@
           <t>April</t>
         </is>
       </c>
-      <c r="C9" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="D9" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="E9" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="F9" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G9" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H9" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="I9" s="24">
+      <c r="C9" s="38" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" s="38" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" s="38" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" s="38" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" s="38" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" s="38" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" s="41">
         <f>SUM(C9:H9)</f>
         <v/>
       </c>
@@ -1714,25 +2416,25 @@
           <t>May</t>
         </is>
       </c>
-      <c r="C10" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="D10" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="E10" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="F10" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G10" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H10" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="I10" s="24">
+      <c r="C10" s="38" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" s="38" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" s="38" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" s="38" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" s="38" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" s="38" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" s="41">
         <f>SUM(C10:H10)</f>
         <v/>
       </c>
@@ -1743,25 +2445,25 @@
           <t>June</t>
         </is>
       </c>
-      <c r="C11" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="D11" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="E11" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="F11" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G11" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H11" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="I11" s="24">
+      <c r="C11" s="38" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" s="38" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" s="38" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" s="38" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" s="38" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" s="38" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" s="41">
         <f>SUM(C11:H11)</f>
         <v/>
       </c>
@@ -1772,25 +2474,25 @@
           <t>July</t>
         </is>
       </c>
-      <c r="C12" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="D12" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="E12" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="F12" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G12" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H12" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="I12" s="24">
+      <c r="C12" s="38" t="n">
+        <v>0</v>
+      </c>
+      <c r="D12" s="38" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" s="38" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" s="38" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" s="38" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" s="38" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" s="41">
         <f>SUM(C12:H12)</f>
         <v/>
       </c>
@@ -1801,25 +2503,25 @@
           <t>August</t>
         </is>
       </c>
-      <c r="C13" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="D13" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="E13" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="F13" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G13" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H13" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="I13" s="24">
+      <c r="C13" s="38" t="n">
+        <v>0</v>
+      </c>
+      <c r="D13" s="38" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" s="38" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" s="38" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" s="38" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" s="38" t="n">
+        <v>0</v>
+      </c>
+      <c r="I13" s="41">
         <f>SUM(C13:H13)</f>
         <v/>
       </c>
@@ -1830,25 +2532,25 @@
           <t>September</t>
         </is>
       </c>
-      <c r="C14" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="D14" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="E14" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="F14" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G14" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H14" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="I14" s="24">
+      <c r="C14" s="38" t="n">
+        <v>0</v>
+      </c>
+      <c r="D14" s="38" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" s="38" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" s="38" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" s="38" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" s="38" t="n">
+        <v>0</v>
+      </c>
+      <c r="I14" s="41">
         <f>SUM(C14:H14)</f>
         <v/>
       </c>
@@ -1859,25 +2561,25 @@
           <t>October</t>
         </is>
       </c>
-      <c r="C15" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="D15" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="E15" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="F15" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G15" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H15" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="I15" s="24">
+      <c r="C15" s="38" t="n">
+        <v>0</v>
+      </c>
+      <c r="D15" s="38" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" s="38" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" s="38" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" s="38" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" s="38" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" s="41">
         <f>SUM(C15:H15)</f>
         <v/>
       </c>
@@ -1888,25 +2590,25 @@
           <t>November</t>
         </is>
       </c>
-      <c r="C16" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="D16" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="E16" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="F16" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G16" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H16" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="I16" s="24">
+      <c r="C16" s="38" t="n">
+        <v>0</v>
+      </c>
+      <c r="D16" s="38" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" s="38" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" s="38" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" s="38" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" s="38" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" s="41">
         <f>SUM(C16:H16)</f>
         <v/>
       </c>
@@ -1917,60 +2619,60 @@
           <t>December</t>
         </is>
       </c>
-      <c r="C17" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="D17" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="E17" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="F17" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G17" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H17" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="I17" s="24">
+      <c r="C17" s="38" t="n">
+        <v>0</v>
+      </c>
+      <c r="D17" s="38" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" s="38" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" s="38" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" s="38" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" s="38" t="n">
+        <v>0</v>
+      </c>
+      <c r="I17" s="41">
         <f>SUM(C17:H17)</f>
         <v/>
       </c>
     </row>
     <row r="18" ht="30" customHeight="1">
-      <c r="B18" s="25" t="inlineStr">
+      <c r="B18" s="42" t="inlineStr">
         <is>
           <t>Annual total</t>
         </is>
       </c>
-      <c r="C18" s="19">
+      <c r="C18" s="37">
         <f>SUM(C6:C17)</f>
         <v/>
       </c>
-      <c r="D18" s="19">
+      <c r="D18" s="37">
         <f>SUM(D6:D17)</f>
         <v/>
       </c>
-      <c r="E18" s="19">
+      <c r="E18" s="37">
         <f>SUM(E6:E17)</f>
         <v/>
       </c>
-      <c r="F18" s="19">
+      <c r="F18" s="37">
         <f>SUM(F6:F17)</f>
         <v/>
       </c>
-      <c r="G18" s="19">
+      <c r="G18" s="37">
         <f>SUM(G6:G17)</f>
         <v/>
       </c>
-      <c r="H18" s="19">
+      <c r="H18" s="37">
         <f>SUM(H6:H17)</f>
         <v/>
       </c>
-      <c r="I18" s="19">
+      <c r="I18" s="37">
         <f>SUM(I6:I17)</f>
         <v/>
       </c>
@@ -2010,7 +2712,7 @@
           <t>Jan–Mar</t>
         </is>
       </c>
-      <c r="D22" s="26">
+      <c r="D22" s="43">
         <f>SUM(I6:I8)</f>
         <v/>
       </c>
@@ -2026,7 +2728,7 @@
           <t>Apr–May</t>
         </is>
       </c>
-      <c r="D23" s="26">
+      <c r="D23" s="43">
         <f>SUM(I9:I10)</f>
         <v/>
       </c>
@@ -2042,7 +2744,7 @@
           <t>Jun–Aug</t>
         </is>
       </c>
-      <c r="D24" s="26">
+      <c r="D24" s="43">
         <f>SUM(I11:I13)</f>
         <v/>
       </c>
@@ -2058,7 +2760,7 @@
           <t>Sep–Dec</t>
         </is>
       </c>
-      <c r="D25" s="26">
+      <c r="D25" s="43">
         <f>SUM(I14:I17)</f>
         <v/>
       </c>
@@ -2074,7 +2776,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2090,7 +2792,7 @@
   </cols>
   <sheetData>
     <row r="2" ht="32" customHeight="1">
-      <c r="B2" s="14" t="inlineStr">
+      <c r="B2" s="34" t="inlineStr">
         <is>
           <t>Tax Calculator</t>
         </is>
@@ -2111,12 +2813,12 @@
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
-      <c r="B6" s="16" t="inlineStr">
+      <c r="B6" s="30" t="inlineStr">
         <is>
           <t>Net SE income (this year)</t>
         </is>
       </c>
-      <c r="C6" s="24">
+      <c r="C6" s="41">
         <f>IF(SEOverride&gt;0,SEOverride,AnnualSEForecast)</f>
         <v/>
       </c>
@@ -2127,12 +2829,12 @@
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
-      <c r="B7" s="16" t="inlineStr">
+      <c r="B7" s="30" t="inlineStr">
         <is>
           <t>× 92.35% (SE tax base)</t>
         </is>
       </c>
-      <c r="C7" s="24">
+      <c r="C7" s="41">
         <f>'Tax Calculator'!$C$6*0.9235</f>
         <v/>
       </c>
@@ -2143,12 +2845,12 @@
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
-      <c r="B8" s="16" t="inlineStr">
+      <c r="B8" s="30" t="inlineStr">
         <is>
           <t>Social Security portion of SE tax (12.4% up to wage base)</t>
         </is>
       </c>
-      <c r="C8" s="24">
+      <c r="C8" s="41">
         <f>MIN('Tax Calculator'!$C$7,SSWageBase)*0.124</f>
         <v/>
       </c>
@@ -2159,12 +2861,12 @@
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="B9" s="16" t="inlineStr">
+      <c r="B9" s="30" t="inlineStr">
         <is>
           <t>Medicare portion of SE tax (2.9%)</t>
         </is>
       </c>
-      <c r="C9" s="24">
+      <c r="C9" s="41">
         <f>'Tax Calculator'!$C$7*0.029</f>
         <v/>
       </c>
@@ -2175,12 +2877,12 @@
       </c>
     </row>
     <row r="10" ht="26" customHeight="1">
-      <c r="B10" s="27" t="inlineStr">
+      <c r="B10" s="44" t="inlineStr">
         <is>
           <t>Total SE tax</t>
         </is>
       </c>
-      <c r="C10" s="28">
+      <c r="C10" s="45">
         <f>'Tax Calculator'!$C$8+'Tax Calculator'!$C$9</f>
         <v/>
       </c>
@@ -2191,12 +2893,12 @@
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">
-      <c r="B11" s="16" t="inlineStr">
+      <c r="B11" s="30" t="inlineStr">
         <is>
           <t>Deductible half of SE tax</t>
         </is>
       </c>
-      <c r="C11" s="24">
+      <c r="C11" s="41">
         <f>'Tax Calculator'!$C$10/2</f>
         <v/>
       </c>
@@ -2214,12 +2916,12 @@
       </c>
     </row>
     <row r="14" ht="22" customHeight="1">
-      <c r="B14" s="16" t="inlineStr">
+      <c r="B14" s="30" t="inlineStr">
         <is>
           <t>AGI (W-2 + net SE − half SE tax)</t>
         </is>
       </c>
-      <c r="C14" s="24">
+      <c r="C14" s="41">
         <f>W2Income+'Tax Calculator'!$C$6-'Tax Calculator'!$C$11</f>
         <v/>
       </c>
@@ -2230,12 +2932,12 @@
       </c>
     </row>
     <row r="15" ht="22" customHeight="1">
-      <c r="B15" s="16" t="inlineStr">
+      <c r="B15" s="30" t="inlineStr">
         <is>
           <t>Standard deduction (based on filing status)</t>
         </is>
       </c>
-      <c r="C15" s="24">
+      <c r="C15" s="41">
         <f>IF(FilingStatus="MFJ",StdDedMFJ,IF(FilingStatus="HOH",StdDedHOH,StdDedSingle))</f>
         <v/>
       </c>
@@ -2246,12 +2948,12 @@
       </c>
     </row>
     <row r="16" ht="22" customHeight="1">
-      <c r="B16" s="16" t="inlineStr">
+      <c r="B16" s="30" t="inlineStr">
         <is>
           <t>Taxable income</t>
         </is>
       </c>
-      <c r="C16" s="24">
+      <c r="C16" s="41">
         <f>MAX('Tax Calculator'!$C$14-'Tax Calculator'!$C$15,0)</f>
         <v/>
       </c>
@@ -2262,12 +2964,12 @@
       </c>
     </row>
     <row r="17" ht="26" customHeight="1">
-      <c r="B17" s="27" t="inlineStr">
+      <c r="B17" s="44" t="inlineStr">
         <is>
           <t>Federal income tax (bracket calc)</t>
         </is>
       </c>
-      <c r="C17" s="28">
+      <c r="C17" s="45">
         <f>IF(FilingStatus="MFJ",SUMPRODUCT(((MIN('Tax Calculator'!$C$16,BracketsMFJ)-IFERROR(OFFSET(BracketsMFJ,-1,0),0))&gt;0)*(MIN('Tax Calculator'!$C$16,BracketsMFJ)-IFERROR(OFFSET(BracketsMFJ,-1,0),0))*BracketsRate),SUMPRODUCT(((MIN('Tax Calculator'!$C$16,BracketsSingle)-IFERROR(OFFSET(BracketsSingle,-1,0),0))&gt;0)*(MIN('Tax Calculator'!$C$16,BracketsSingle)-IFERROR(OFFSET(BracketsSingle,-1,0),0))*BracketsRate))</f>
         <v/>
       </c>
@@ -2285,12 +2987,12 @@
       </c>
     </row>
     <row r="20" ht="26" customHeight="1">
-      <c r="B20" s="27" t="inlineStr">
+      <c r="B20" s="44" t="inlineStr">
         <is>
           <t>State income tax (flat rate × taxable income)</t>
         </is>
       </c>
-      <c r="C20" s="28">
+      <c r="C20" s="45">
         <f>'Tax Calculator'!$C$16*StateRate</f>
         <v/>
       </c>
@@ -2301,12 +3003,12 @@
       </c>
     </row>
     <row r="21" ht="22" customHeight="1">
-      <c r="B21" s="16" t="inlineStr">
+      <c r="B21" s="30" t="inlineStr">
         <is>
           <t>Total federal owed (SE + income)</t>
         </is>
       </c>
-      <c r="C21" s="24">
+      <c r="C21" s="41">
         <f>'Tax Calculator'!$C$10+'Tax Calculator'!$C$17</f>
         <v/>
       </c>
@@ -2317,12 +3019,12 @@
       </c>
     </row>
     <row r="22" ht="22" customHeight="1">
-      <c r="B22" s="16" t="inlineStr">
+      <c r="B22" s="30" t="inlineStr">
         <is>
           <t>Less: W-2 federal withholding</t>
         </is>
       </c>
-      <c r="C22" s="24">
+      <c r="C22" s="41">
         <f>-W2Withheld</f>
         <v/>
       </c>
@@ -2333,11 +3035,11 @@
       </c>
     </row>
     <row r="23" ht="26" customHeight="1">
-      <c r="B23" s="27">
+      <c r="B23" s="44">
         <f> Net federal owed (quarterly target)</f>
         <v/>
       </c>
-      <c r="C23" s="28">
+      <c r="C23" s="45">
         <f>'Tax Calculator'!$C$21-W2Withheld</f>
         <v/>
       </c>
@@ -2348,12 +3050,12 @@
       </c>
     </row>
     <row r="24" ht="26" customHeight="1">
-      <c r="B24" s="27" t="inlineStr">
+      <c r="B24" s="44" t="inlineStr">
         <is>
           <t>Total state owed (quarterly target)</t>
         </is>
       </c>
-      <c r="C24" s="28">
+      <c r="C24" s="45">
         <f>'Tax Calculator'!$C$20</f>
         <v/>
       </c>
@@ -2375,7 +3077,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2395,7 +3097,7 @@
   </cols>
   <sheetData>
     <row r="2" ht="32" customHeight="1">
-      <c r="B2" s="14" t="inlineStr">
+      <c r="B2" s="34" t="inlineStr">
         <is>
           <t>Quarterly Payments</t>
         </is>
@@ -2416,37 +3118,37 @@
       </c>
     </row>
     <row r="6" ht="24" customHeight="1">
-      <c r="B6" s="29" t="inlineStr">
+      <c r="B6" s="46" t="inlineStr">
         <is>
           <t>Q</t>
         </is>
       </c>
-      <c r="C6" s="29" t="inlineStr">
+      <c r="C6" s="46" t="inlineStr">
         <is>
           <t>Due date</t>
         </is>
       </c>
-      <c r="D6" s="29" t="inlineStr">
+      <c r="D6" s="46" t="inlineStr">
         <is>
           <t>Target $</t>
         </is>
       </c>
-      <c r="E6" s="29" t="inlineStr">
+      <c r="E6" s="46" t="inlineStr">
         <is>
           <t>Paid date</t>
         </is>
       </c>
-      <c r="F6" s="29" t="inlineStr">
+      <c r="F6" s="46" t="inlineStr">
         <is>
           <t>Paid $</t>
         </is>
       </c>
-      <c r="G6" s="29" t="inlineStr">
+      <c r="G6" s="46" t="inlineStr">
         <is>
           <t>Method</t>
         </is>
       </c>
-      <c r="H6" s="29" t="inlineStr">
+      <c r="H6" s="46" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
@@ -2463,13 +3165,13 @@
           <t>April 15</t>
         </is>
       </c>
-      <c r="D7" s="24">
+      <c r="D7" s="41">
         <f>NetFedOwed/4</f>
         <v/>
       </c>
-      <c r="E7" s="30" t="n"/>
-      <c r="F7" s="20" t="n"/>
-      <c r="G7" s="31" t="n"/>
+      <c r="E7" s="47" t="n"/>
+      <c r="F7" s="38" t="n"/>
+      <c r="G7" s="48" t="n"/>
       <c r="H7" s="10">
         <f>IF(F7="","Not paid yet",IF(F7&gt;=D7*0.95,"On track","Underpaid by $"&amp;TEXT(D7-F7,"#,##0")))</f>
         <v/>
@@ -2486,13 +3188,13 @@
           <t>June 15</t>
         </is>
       </c>
-      <c r="D8" s="24">
+      <c r="D8" s="41">
         <f>NetFedOwed/4</f>
         <v/>
       </c>
-      <c r="E8" s="30" t="n"/>
-      <c r="F8" s="20" t="n"/>
-      <c r="G8" s="31" t="n"/>
+      <c r="E8" s="47" t="n"/>
+      <c r="F8" s="38" t="n"/>
+      <c r="G8" s="48" t="n"/>
       <c r="H8" s="10">
         <f>IF(F8="","Not paid yet",IF(F8&gt;=D8*0.95,"On track","Underpaid by $"&amp;TEXT(D8-F8,"#,##0")))</f>
         <v/>
@@ -2509,13 +3211,13 @@
           <t>September 15</t>
         </is>
       </c>
-      <c r="D9" s="24">
+      <c r="D9" s="41">
         <f>NetFedOwed/4</f>
         <v/>
       </c>
-      <c r="E9" s="30" t="n"/>
-      <c r="F9" s="20" t="n"/>
-      <c r="G9" s="31" t="n"/>
+      <c r="E9" s="47" t="n"/>
+      <c r="F9" s="38" t="n"/>
+      <c r="G9" s="48" t="n"/>
       <c r="H9" s="10">
         <f>IF(F9="","Not paid yet",IF(F9&gt;=D9*0.95,"On track","Underpaid by $"&amp;TEXT(D9-F9,"#,##0")))</f>
         <v/>
@@ -2532,34 +3234,34 @@
           <t>January 15</t>
         </is>
       </c>
-      <c r="D10" s="24">
+      <c r="D10" s="41">
         <f>NetFedOwed/4</f>
         <v/>
       </c>
-      <c r="E10" s="30" t="n"/>
-      <c r="F10" s="20" t="n"/>
-      <c r="G10" s="31" t="n"/>
+      <c r="E10" s="47" t="n"/>
+      <c r="F10" s="38" t="n"/>
+      <c r="G10" s="48" t="n"/>
       <c r="H10" s="10">
         <f>IF(F10="","Not paid yet",IF(F10&gt;=D10*0.95,"On track","Underpaid by $"&amp;TEXT(D10-F10,"#,##0")))</f>
         <v/>
       </c>
     </row>
     <row r="11" ht="28" customHeight="1">
-      <c r="B11" s="25" t="inlineStr">
+      <c r="B11" s="42" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="C11" s="32" t="n"/>
-      <c r="D11" s="19">
+      <c r="C11" s="49" t="n"/>
+      <c r="D11" s="37">
         <f>SUM(D7:D10)</f>
         <v/>
       </c>
-      <c r="F11" s="19">
+      <c r="F11" s="37">
         <f>SUM(F7:F10)</f>
         <v/>
       </c>
-      <c r="H11" s="25">
+      <c r="H11" s="42">
         <f>IF(F11&gt;=D11*0.95,"Annual target met","Short $"&amp;TEXT(D11-F11,"#,##0"))</f>
         <v/>
       </c>
@@ -2572,37 +3274,37 @@
       </c>
     </row>
     <row r="15" ht="24" customHeight="1">
-      <c r="B15" s="29" t="inlineStr">
+      <c r="B15" s="46" t="inlineStr">
         <is>
           <t>Q</t>
         </is>
       </c>
-      <c r="C15" s="29" t="inlineStr">
+      <c r="C15" s="46" t="inlineStr">
         <is>
           <t>Due date</t>
         </is>
       </c>
-      <c r="D15" s="29" t="inlineStr">
+      <c r="D15" s="46" t="inlineStr">
         <is>
           <t>Target $</t>
         </is>
       </c>
-      <c r="E15" s="29" t="inlineStr">
+      <c r="E15" s="46" t="inlineStr">
         <is>
           <t>Paid date</t>
         </is>
       </c>
-      <c r="F15" s="29" t="inlineStr">
+      <c r="F15" s="46" t="inlineStr">
         <is>
           <t>Paid $</t>
         </is>
       </c>
-      <c r="G15" s="29" t="inlineStr">
+      <c r="G15" s="46" t="inlineStr">
         <is>
           <t>Method</t>
         </is>
       </c>
-      <c r="H15" s="29" t="inlineStr">
+      <c r="H15" s="46" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
@@ -2619,13 +3321,13 @@
           <t>April 15</t>
         </is>
       </c>
-      <c r="D16" s="24">
+      <c r="D16" s="41">
         <f>NetStateOwed/4</f>
         <v/>
       </c>
-      <c r="E16" s="30" t="n"/>
-      <c r="F16" s="20" t="n"/>
-      <c r="G16" s="31" t="n"/>
+      <c r="E16" s="47" t="n"/>
+      <c r="F16" s="38" t="n"/>
+      <c r="G16" s="48" t="n"/>
       <c r="H16" s="10">
         <f>IF(F16="","Not paid yet",IF(F16&gt;=D16*0.95,"On track","Underpaid by $"&amp;TEXT(D16-F16,"#,##0")))</f>
         <v/>
@@ -2642,13 +3344,13 @@
           <t>June 15</t>
         </is>
       </c>
-      <c r="D17" s="24">
+      <c r="D17" s="41">
         <f>NetStateOwed/4</f>
         <v/>
       </c>
-      <c r="E17" s="30" t="n"/>
-      <c r="F17" s="20" t="n"/>
-      <c r="G17" s="31" t="n"/>
+      <c r="E17" s="47" t="n"/>
+      <c r="F17" s="38" t="n"/>
+      <c r="G17" s="48" t="n"/>
       <c r="H17" s="10">
         <f>IF(F17="","Not paid yet",IF(F17&gt;=D17*0.95,"On track","Underpaid by $"&amp;TEXT(D17-F17,"#,##0")))</f>
         <v/>
@@ -2665,13 +3367,13 @@
           <t>September 15</t>
         </is>
       </c>
-      <c r="D18" s="24">
+      <c r="D18" s="41">
         <f>NetStateOwed/4</f>
         <v/>
       </c>
-      <c r="E18" s="30" t="n"/>
-      <c r="F18" s="20" t="n"/>
-      <c r="G18" s="31" t="n"/>
+      <c r="E18" s="47" t="n"/>
+      <c r="F18" s="38" t="n"/>
+      <c r="G18" s="48" t="n"/>
       <c r="H18" s="10">
         <f>IF(F18="","Not paid yet",IF(F18&gt;=D18*0.95,"On track","Underpaid by $"&amp;TEXT(D18-F18,"#,##0")))</f>
         <v/>
@@ -2688,30 +3390,30 @@
           <t>January 15</t>
         </is>
       </c>
-      <c r="D19" s="24">
+      <c r="D19" s="41">
         <f>NetStateOwed/4</f>
         <v/>
       </c>
-      <c r="E19" s="30" t="n"/>
-      <c r="F19" s="20" t="n"/>
-      <c r="G19" s="31" t="n"/>
+      <c r="E19" s="47" t="n"/>
+      <c r="F19" s="38" t="n"/>
+      <c r="G19" s="48" t="n"/>
       <c r="H19" s="10">
         <f>IF(F19="","Not paid yet",IF(F19&gt;=D19*0.95,"On track","Underpaid by $"&amp;TEXT(D19-F19,"#,##0")))</f>
         <v/>
       </c>
     </row>
     <row r="20" ht="28" customHeight="1">
-      <c r="B20" s="25" t="inlineStr">
+      <c r="B20" s="42" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="C20" s="32" t="n"/>
-      <c r="D20" s="19">
+      <c r="C20" s="49" t="n"/>
+      <c r="D20" s="37">
         <f>SUM(D16:D19)</f>
         <v/>
       </c>
-      <c r="F20" s="19">
+      <c r="F20" s="37">
         <f>SUM(F16:F19)</f>
         <v/>
       </c>
@@ -2726,98 +3428,98 @@
     <mergeCell ref="B5:H5"/>
   </mergeCells>
   <conditionalFormatting sqref="H7">
-    <cfRule type="expression" priority="1" dxfId="0">
+    <cfRule type="expression" priority="1" dxfId="2">
       <formula>ISNUMBER(SEARCH("On track",H7))</formula>
     </cfRule>
-    <cfRule type="expression" priority="2" dxfId="1">
+    <cfRule type="expression" priority="2" dxfId="3">
       <formula>ISNUMBER(SEARCH("Not paid",H7))</formula>
     </cfRule>
-    <cfRule type="expression" priority="3" dxfId="2">
+    <cfRule type="expression" priority="3" dxfId="4">
       <formula>ISNUMBER(SEARCH("Underpaid",H7))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H8">
-    <cfRule type="expression" priority="4" dxfId="0">
+    <cfRule type="expression" priority="4" dxfId="2">
       <formula>ISNUMBER(SEARCH("On track",H8))</formula>
     </cfRule>
-    <cfRule type="expression" priority="5" dxfId="1">
+    <cfRule type="expression" priority="5" dxfId="3">
       <formula>ISNUMBER(SEARCH("Not paid",H8))</formula>
     </cfRule>
-    <cfRule type="expression" priority="6" dxfId="2">
+    <cfRule type="expression" priority="6" dxfId="4">
       <formula>ISNUMBER(SEARCH("Underpaid",H8))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H9">
-    <cfRule type="expression" priority="7" dxfId="0">
+    <cfRule type="expression" priority="7" dxfId="2">
       <formula>ISNUMBER(SEARCH("On track",H9))</formula>
     </cfRule>
-    <cfRule type="expression" priority="8" dxfId="1">
+    <cfRule type="expression" priority="8" dxfId="3">
       <formula>ISNUMBER(SEARCH("Not paid",H9))</formula>
     </cfRule>
-    <cfRule type="expression" priority="9" dxfId="2">
+    <cfRule type="expression" priority="9" dxfId="4">
       <formula>ISNUMBER(SEARCH("Underpaid",H9))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H10">
-    <cfRule type="expression" priority="10" dxfId="0">
+    <cfRule type="expression" priority="10" dxfId="2">
       <formula>ISNUMBER(SEARCH("On track",H10))</formula>
     </cfRule>
-    <cfRule type="expression" priority="11" dxfId="1">
+    <cfRule type="expression" priority="11" dxfId="3">
       <formula>ISNUMBER(SEARCH("Not paid",H10))</formula>
     </cfRule>
-    <cfRule type="expression" priority="12" dxfId="2">
+    <cfRule type="expression" priority="12" dxfId="4">
       <formula>ISNUMBER(SEARCH("Underpaid",H10))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H11">
-    <cfRule type="expression" priority="13" dxfId="0">
+    <cfRule type="expression" priority="13" dxfId="2">
       <formula>ISNUMBER(SEARCH("met",H11))</formula>
     </cfRule>
-    <cfRule type="expression" priority="14" dxfId="2">
+    <cfRule type="expression" priority="14" dxfId="4">
       <formula>ISNUMBER(SEARCH("Short",H11))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H16">
-    <cfRule type="expression" priority="15" dxfId="0">
+    <cfRule type="expression" priority="15" dxfId="2">
       <formula>ISNUMBER(SEARCH("On track",H16))</formula>
     </cfRule>
-    <cfRule type="expression" priority="16" dxfId="1">
+    <cfRule type="expression" priority="16" dxfId="3">
       <formula>ISNUMBER(SEARCH("Not paid",H16))</formula>
     </cfRule>
-    <cfRule type="expression" priority="17" dxfId="2">
+    <cfRule type="expression" priority="17" dxfId="4">
       <formula>ISNUMBER(SEARCH("Underpaid",H16))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H17">
-    <cfRule type="expression" priority="18" dxfId="0">
+    <cfRule type="expression" priority="18" dxfId="2">
       <formula>ISNUMBER(SEARCH("On track",H17))</formula>
     </cfRule>
-    <cfRule type="expression" priority="19" dxfId="1">
+    <cfRule type="expression" priority="19" dxfId="3">
       <formula>ISNUMBER(SEARCH("Not paid",H17))</formula>
     </cfRule>
-    <cfRule type="expression" priority="20" dxfId="2">
+    <cfRule type="expression" priority="20" dxfId="4">
       <formula>ISNUMBER(SEARCH("Underpaid",H17))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H18">
-    <cfRule type="expression" priority="21" dxfId="0">
+    <cfRule type="expression" priority="21" dxfId="2">
       <formula>ISNUMBER(SEARCH("On track",H18))</formula>
     </cfRule>
-    <cfRule type="expression" priority="22" dxfId="1">
+    <cfRule type="expression" priority="22" dxfId="3">
       <formula>ISNUMBER(SEARCH("Not paid",H18))</formula>
     </cfRule>
-    <cfRule type="expression" priority="23" dxfId="2">
+    <cfRule type="expression" priority="23" dxfId="4">
       <formula>ISNUMBER(SEARCH("Underpaid",H18))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H19">
-    <cfRule type="expression" priority="24" dxfId="0">
+    <cfRule type="expression" priority="24" dxfId="2">
       <formula>ISNUMBER(SEARCH("On track",H19))</formula>
     </cfRule>
-    <cfRule type="expression" priority="25" dxfId="1">
+    <cfRule type="expression" priority="25" dxfId="3">
       <formula>ISNUMBER(SEARCH("Not paid",H19))</formula>
     </cfRule>
-    <cfRule type="expression" priority="26" dxfId="2">
+    <cfRule type="expression" priority="26" dxfId="4">
       <formula>ISNUMBER(SEARCH("Underpaid",H19))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -2825,7 +3527,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2841,7 +3543,7 @@
   </cols>
   <sheetData>
     <row r="2" ht="32" customHeight="1">
-      <c r="B2" s="14" t="inlineStr">
+      <c r="B2" s="34" t="inlineStr">
         <is>
           <t>Safe Harbor Check</t>
         </is>
@@ -2862,12 +3564,12 @@
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
-      <c r="B6" s="16" t="inlineStr">
+      <c r="B6" s="30" t="inlineStr">
         <is>
           <t>Required multiplier (110% if last year AGI &gt; $150K, else 100%)</t>
         </is>
       </c>
-      <c r="C6" s="33">
+      <c r="C6" s="50">
         <f>IF(LastYearAGI&gt;150000,1.1,1)</f>
         <v/>
       </c>
@@ -2878,12 +3580,12 @@
       </c>
     </row>
     <row r="7" ht="26" customHeight="1">
-      <c r="B7" s="27" t="inlineStr">
+      <c r="B7" s="44" t="inlineStr">
         <is>
           <t>Safe harbor target (last year's tax × multiplier)</t>
         </is>
       </c>
-      <c r="C7" s="19">
+      <c r="C7" s="37">
         <f>LastYearTax*C6</f>
         <v/>
       </c>
@@ -2894,12 +3596,12 @@
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
-      <c r="B8" s="16" t="inlineStr">
+      <c r="B8" s="30" t="inlineStr">
         <is>
           <t>Paid so far (Q1–Q4 federal + W-2 withholding)</t>
         </is>
       </c>
-      <c r="C8" s="24">
+      <c r="C8" s="41">
         <f>FedPaidYTD+W2Withheld</f>
         <v/>
       </c>
@@ -2910,12 +3612,12 @@
       </c>
     </row>
     <row r="9" ht="32" customHeight="1">
-      <c r="B9" s="27" t="inlineStr">
+      <c r="B9" s="44" t="inlineStr">
         <is>
           <t>Safe Harbor 1 status:</t>
         </is>
       </c>
-      <c r="C9" s="34">
+      <c r="C9" s="51">
         <f>IF(C8&gt;=C7,"✓ SAFE","Short $"&amp;TEXT(C7-C8,"#,##0"))</f>
         <v/>
       </c>
@@ -2928,12 +3630,12 @@
       </c>
     </row>
     <row r="12" ht="22" customHeight="1">
-      <c r="B12" s="16" t="inlineStr">
+      <c r="B12" s="30" t="inlineStr">
         <is>
           <t>This year's projected total federal tax</t>
         </is>
       </c>
-      <c r="C12" s="24">
+      <c r="C12" s="41">
         <f>TotalFedTax</f>
         <v/>
       </c>
@@ -2944,12 +3646,12 @@
       </c>
     </row>
     <row r="13" ht="26" customHeight="1">
-      <c r="B13" s="27" t="inlineStr">
+      <c r="B13" s="44" t="inlineStr">
         <is>
           <t>Safe harbor target (90% of this year's tax)</t>
         </is>
       </c>
-      <c r="C13" s="19">
+      <c r="C13" s="37">
         <f>C12*0.9</f>
         <v/>
       </c>
@@ -2960,12 +3662,12 @@
       </c>
     </row>
     <row r="14" ht="22" customHeight="1">
-      <c r="B14" s="16" t="inlineStr">
+      <c r="B14" s="30" t="inlineStr">
         <is>
           <t>Paid so far (Q1–Q4 federal + W-2 withholding)</t>
         </is>
       </c>
-      <c r="C14" s="24">
+      <c r="C14" s="41">
         <f>FedPaidYTD+W2Withheld</f>
         <v/>
       </c>
@@ -2976,12 +3678,12 @@
       </c>
     </row>
     <row r="15" ht="32" customHeight="1">
-      <c r="B15" s="27" t="inlineStr">
+      <c r="B15" s="44" t="inlineStr">
         <is>
           <t>Safe Harbor 2 status:</t>
         </is>
       </c>
-      <c r="C15" s="34">
+      <c r="C15" s="51">
         <f>IF(C14&gt;=C13,"✓ SAFE","Short $"&amp;TEXT(C13-C14,"#,##0"))</f>
         <v/>
       </c>
@@ -2994,12 +3696,12 @@
       </c>
     </row>
     <row r="18" ht="38" customHeight="1">
-      <c r="B18" s="27" t="inlineStr">
+      <c r="B18" s="44" t="inlineStr">
         <is>
           <t>Overall status:</t>
         </is>
       </c>
-      <c r="C18" s="34">
+      <c r="C18" s="51">
         <f>IF(OR(C8&gt;=C7,C14&gt;=C13),"✓ YES — you're safe from penalty","⚠ Not yet — close one of the gaps above")</f>
         <v/>
       </c>
@@ -3021,26 +3723,26 @@
     <mergeCell ref="B20:D20"/>
   </mergeCells>
   <conditionalFormatting sqref="C9">
-    <cfRule type="expression" priority="1" dxfId="3">
+    <cfRule type="expression" priority="1" dxfId="5">
       <formula>ISNUMBER(SEARCH("SAFE",C9))</formula>
     </cfRule>
-    <cfRule type="expression" priority="2" dxfId="4">
+    <cfRule type="expression" priority="2" dxfId="6">
       <formula>ISNUMBER(SEARCH("Short",C9))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C15">
-    <cfRule type="expression" priority="3" dxfId="3">
+    <cfRule type="expression" priority="3" dxfId="5">
       <formula>ISNUMBER(SEARCH("SAFE",C15))</formula>
     </cfRule>
-    <cfRule type="expression" priority="4" dxfId="4">
+    <cfRule type="expression" priority="4" dxfId="6">
       <formula>ISNUMBER(SEARCH("Short",C15))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C18">
-    <cfRule type="expression" priority="5" dxfId="3">
+    <cfRule type="expression" priority="5" dxfId="5">
       <formula>ISNUMBER(SEARCH("YES",C18))</formula>
     </cfRule>
-    <cfRule type="expression" priority="6" dxfId="5">
+    <cfRule type="expression" priority="6" dxfId="7">
       <formula>ISNUMBER(SEARCH("Not yet",C18))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3048,7 +3750,553 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B2:E42"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="2" customWidth="1" min="1" max="1"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="2" ht="32" customHeight="1">
+      <c r="B2" s="34" t="inlineStr">
+        <is>
+          <t>Worked Examples</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" s="15" t="inlineStr">
+        <is>
+          <t>Three real scenarios showing exactly what numbers go where. Compare to your own situation, then plug yours into the Setup tab.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="28" customHeight="1">
+      <c r="B5" s="52" t="inlineStr"/>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>DoorDash full-timer</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>Freelancer + W-2 day job</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>Etsy seller</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="68" customHeight="1">
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>Situation</t>
+        </is>
+      </c>
+      <c r="C6" s="53" t="inlineStr">
+        <is>
+          <t>Single, lives in CA, Dashes full time. Tracked 22,000 business miles. Gross earnings $58,000 minus $15,400 mileage deduction = $42,600 net.</t>
+        </is>
+      </c>
+      <c r="D6" s="53" t="inlineStr">
+        <is>
+          <t>MFJ, NY, $48K W-2 day job with $5,400 federal withholding + $60K net freelance design work on the side.</t>
+        </is>
+      </c>
+      <c r="E6" s="53" t="inlineStr">
+        <is>
+          <t>Single, TX (no state tax), Etsy print shop. $25,000 net profit after COGS and home office deduction.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="24" customHeight="1">
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Setup tab inputs</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="22" customHeight="1">
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>Filing status</t>
+        </is>
+      </c>
+      <c r="C9" s="54" t="inlineStr">
+        <is>
+          <t>Single</t>
+        </is>
+      </c>
+      <c r="D9" s="54" t="inlineStr">
+        <is>
+          <t>MFJ</t>
+        </is>
+      </c>
+      <c r="E9" s="54" t="inlineStr">
+        <is>
+          <t>Single</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="22" customHeight="1">
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>State</t>
+        </is>
+      </c>
+      <c r="C10" s="54" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="D10" s="54" t="inlineStr">
+        <is>
+          <t>NY</t>
+        </is>
+      </c>
+      <c r="E10" s="54" t="inlineStr">
+        <is>
+          <t>TX</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="22" customHeight="1">
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>State flat estimated tax rate</t>
+        </is>
+      </c>
+      <c r="C11" s="55" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="D11" s="55" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="E11" s="55" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" ht="22" customHeight="1">
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>Net SE income (annual)</t>
+        </is>
+      </c>
+      <c r="C12" s="56" t="n">
+        <v>42600</v>
+      </c>
+      <c r="D12" s="56" t="n">
+        <v>60000</v>
+      </c>
+      <c r="E12" s="56" t="n">
+        <v>25000</v>
+      </c>
+    </row>
+    <row r="13" ht="22" customHeight="1">
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>W-2 income</t>
+        </is>
+      </c>
+      <c r="C13" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="D13" s="56" t="n">
+        <v>48000</v>
+      </c>
+      <c r="E13" s="56" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" ht="22" customHeight="1">
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>Federal tax withheld from W-2</t>
+        </is>
+      </c>
+      <c r="C14" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="D14" s="56" t="n">
+        <v>5400</v>
+      </c>
+      <c r="E14" s="56" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" ht="22" customHeight="1">
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>Last year's total federal tax</t>
+        </is>
+      </c>
+      <c r="C15" s="56" t="n">
+        <v>3200</v>
+      </c>
+      <c r="D15" s="56" t="n">
+        <v>8900</v>
+      </c>
+      <c r="E15" s="56" t="n">
+        <v>1800</v>
+      </c>
+    </row>
+    <row r="16" ht="22" customHeight="1">
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>Last year's AGI</t>
+        </is>
+      </c>
+      <c r="C16" s="56" t="n">
+        <v>38000</v>
+      </c>
+      <c r="D16" s="56" t="n">
+        <v>98000</v>
+      </c>
+      <c r="E16" s="56" t="n">
+        <v>24000</v>
+      </c>
+    </row>
+    <row r="18" ht="24" customHeight="1">
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>What the Tax Calculator returns</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="22" customHeight="1">
+      <c r="B19" s="9" t="inlineStr">
+        <is>
+          <t>Net SE income × 92.35% (SE base)</t>
+        </is>
+      </c>
+      <c r="C19" s="56" t="n">
+        <v>39341</v>
+      </c>
+      <c r="D19" s="56" t="n">
+        <v>55410</v>
+      </c>
+      <c r="E19" s="56" t="n">
+        <v>23088</v>
+      </c>
+    </row>
+    <row r="20" ht="22" customHeight="1">
+      <c r="B20" s="9" t="inlineStr">
+        <is>
+          <t>Social Security (12.4%)</t>
+        </is>
+      </c>
+      <c r="C20" s="56" t="n">
+        <v>4878</v>
+      </c>
+      <c r="D20" s="56" t="n">
+        <v>6871</v>
+      </c>
+      <c r="E20" s="56" t="n">
+        <v>2863</v>
+      </c>
+    </row>
+    <row r="21" ht="22" customHeight="1">
+      <c r="B21" s="9" t="inlineStr">
+        <is>
+          <t>Medicare (2.9%)</t>
+        </is>
+      </c>
+      <c r="C21" s="56" t="n">
+        <v>1141</v>
+      </c>
+      <c r="D21" s="56" t="n">
+        <v>1607</v>
+      </c>
+      <c r="E21" s="56" t="n">
+        <v>669</v>
+      </c>
+    </row>
+    <row r="22" ht="22" customHeight="1">
+      <c r="B22" s="57" t="inlineStr">
+        <is>
+          <t>Total SE tax</t>
+        </is>
+      </c>
+      <c r="C22" s="45" t="n">
+        <v>6019</v>
+      </c>
+      <c r="D22" s="45" t="n">
+        <v>8478</v>
+      </c>
+      <c r="E22" s="45" t="n">
+        <v>3532</v>
+      </c>
+    </row>
+    <row r="23" ht="22" customHeight="1">
+      <c r="B23" s="9" t="inlineStr">
+        <is>
+          <t>AGI (W-2 + net SE − ½ SE tax)</t>
+        </is>
+      </c>
+      <c r="C23" s="56" t="n">
+        <v>39591</v>
+      </c>
+      <c r="D23" s="56" t="n">
+        <v>103761</v>
+      </c>
+      <c r="E23" s="56" t="n">
+        <v>23234</v>
+      </c>
+    </row>
+    <row r="24" ht="22" customHeight="1">
+      <c r="B24" s="9" t="inlineStr">
+        <is>
+          <t>Standard deduction</t>
+        </is>
+      </c>
+      <c r="C24" s="56" t="n">
+        <v>15750</v>
+      </c>
+      <c r="D24" s="56" t="n">
+        <v>31500</v>
+      </c>
+      <c r="E24" s="56" t="n">
+        <v>15750</v>
+      </c>
+    </row>
+    <row r="25" ht="22" customHeight="1">
+      <c r="B25" s="9" t="inlineStr">
+        <is>
+          <t>Taxable income</t>
+        </is>
+      </c>
+      <c r="C25" s="56" t="n">
+        <v>23841</v>
+      </c>
+      <c r="D25" s="56" t="n">
+        <v>72261</v>
+      </c>
+      <c r="E25" s="56" t="n">
+        <v>7484</v>
+      </c>
+    </row>
+    <row r="26" ht="22" customHeight="1">
+      <c r="B26" s="57" t="inlineStr">
+        <is>
+          <t>Federal income tax (bracket calc)</t>
+        </is>
+      </c>
+      <c r="C26" s="45" t="n">
+        <v>2622</v>
+      </c>
+      <c r="D26" s="45" t="n">
+        <v>8195</v>
+      </c>
+      <c r="E26" s="45" t="n">
+        <v>748</v>
+      </c>
+    </row>
+    <row r="27" ht="22" customHeight="1">
+      <c r="B27" s="57" t="inlineStr">
+        <is>
+          <t>State income tax</t>
+        </is>
+      </c>
+      <c r="C27" s="45" t="n">
+        <v>1430</v>
+      </c>
+      <c r="D27" s="45" t="n">
+        <v>3613</v>
+      </c>
+      <c r="E27" s="45" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" ht="24" customHeight="1">
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>What you'd pay each quarter</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="22" customHeight="1">
+      <c r="B30" s="9" t="inlineStr">
+        <is>
+          <t>Total federal owed (SE + income tax)</t>
+        </is>
+      </c>
+      <c r="C30" s="56" t="n">
+        <v>8641</v>
+      </c>
+      <c r="D30" s="56" t="n">
+        <v>16673</v>
+      </c>
+      <c r="E30" s="56" t="n">
+        <v>4280</v>
+      </c>
+    </row>
+    <row r="31" ht="22" customHeight="1">
+      <c r="B31" s="9" t="inlineStr">
+        <is>
+          <t>Less: W-2 federal withholding</t>
+        </is>
+      </c>
+      <c r="C31" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="D31" s="56" t="n">
+        <v>-5400</v>
+      </c>
+      <c r="E31" s="56" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" ht="22" customHeight="1">
+      <c r="B32" s="57" t="inlineStr">
+        <is>
+          <t>Net federal owed (quarterly target ÷ 4)</t>
+        </is>
+      </c>
+      <c r="C32" s="45" t="n">
+        <v>8641</v>
+      </c>
+      <c r="D32" s="45" t="n">
+        <v>11273</v>
+      </c>
+      <c r="E32" s="45" t="n">
+        <v>4280</v>
+      </c>
+    </row>
+    <row r="33" ht="22" customHeight="1">
+      <c r="B33" s="57" t="inlineStr">
+        <is>
+          <t>Each federal quarterly payment</t>
+        </is>
+      </c>
+      <c r="C33" s="45" t="n">
+        <v>2160</v>
+      </c>
+      <c r="D33" s="45" t="n">
+        <v>2818</v>
+      </c>
+      <c r="E33" s="45" t="n">
+        <v>1070</v>
+      </c>
+    </row>
+    <row r="34" ht="22" customHeight="1">
+      <c r="B34" s="57" t="inlineStr">
+        <is>
+          <t>Each state quarterly payment</t>
+        </is>
+      </c>
+      <c r="C34" s="45" t="n">
+        <v>358</v>
+      </c>
+      <c r="D34" s="45" t="n">
+        <v>903</v>
+      </c>
+      <c r="E34" s="45" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" ht="24" customHeight="1">
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>Safe Harbor target (whichever is lower wins)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="22" customHeight="1">
+      <c r="B37" s="9" t="inlineStr">
+        <is>
+          <t>100% of last year's tax (110% if AGI &gt; $150K)</t>
+        </is>
+      </c>
+      <c r="C37" s="56" t="n">
+        <v>3200</v>
+      </c>
+      <c r="D37" s="56" t="n">
+        <v>8900</v>
+      </c>
+      <c r="E37" s="56" t="n">
+        <v>1800</v>
+      </c>
+    </row>
+    <row r="38" ht="22" customHeight="1">
+      <c r="B38" s="9" t="inlineStr">
+        <is>
+          <t>90% of this year's projected tax</t>
+        </is>
+      </c>
+      <c r="C38" s="56" t="n">
+        <v>7777</v>
+      </c>
+      <c r="D38" s="56" t="n">
+        <v>15006</v>
+      </c>
+      <c r="E38" s="56" t="n">
+        <v>3852</v>
+      </c>
+    </row>
+    <row r="39" ht="22" customHeight="1">
+      <c r="B39" s="57" t="inlineStr">
+        <is>
+          <t>Easier safe harbor — total to pay across 4 quarters</t>
+        </is>
+      </c>
+      <c r="C39" s="45" t="n">
+        <v>3200</v>
+      </c>
+      <c r="D39" s="45" t="n">
+        <v>8900</v>
+      </c>
+      <c r="E39" s="45" t="n">
+        <v>1800</v>
+      </c>
+    </row>
+    <row r="40" ht="22" customHeight="1">
+      <c r="B40" s="57">
+        <f> safe-harbor quarterly amount</f>
+        <v/>
+      </c>
+      <c r="C40" s="45" t="n">
+        <v>800</v>
+      </c>
+      <c r="D40" s="45" t="n">
+        <v>2225</v>
+      </c>
+      <c r="E40" s="45" t="n">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="42" ht="70" customHeight="1">
+      <c r="B42" s="4" t="inlineStr">
+        <is>
+          <t>Notice the difference: paying TRUE this-year tax is the conservative play (more cash out now, no April surprise). Paying SAFE-HARBOR is the minimum to avoid the penalty (lower quarterly checks, but you'll owe a balance in April). Both are valid. Most people pick safe-harbor for cash-flow reasons. The Quarterly Payments tab targets the TRUE number; drop it down to the safe-harbor number if cash is tight.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="7">
+    <mergeCell ref="B18:E18"/>
+    <mergeCell ref="B8:E8"/>
+    <mergeCell ref="B29:E29"/>
+    <mergeCell ref="B3:E3"/>
+    <mergeCell ref="B2:E2"/>
+    <mergeCell ref="B42:E42"/>
+    <mergeCell ref="B36:E36"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3063,7 +4311,7 @@
   </cols>
   <sheetData>
     <row r="2" ht="32" customHeight="1">
-      <c r="B2" s="14" t="inlineStr">
+      <c r="B2" s="34" t="inlineStr">
         <is>
           <t>IRS &amp; State Quarterly Tax Reference</t>
         </is>
@@ -3077,12 +4325,12 @@
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
-      <c r="B5" s="35" t="inlineStr">
+      <c r="B5" s="58" t="inlineStr">
         <is>
           <t>Q</t>
         </is>
       </c>
-      <c r="C5" s="27" t="inlineStr">
+      <c r="C5" s="44" t="inlineStr">
         <is>
           <t>Where do I actually pay federal quarterly tax?</t>
         </is>
@@ -3096,12 +4344,12 @@
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
-      <c r="B8" s="35" t="inlineStr">
+      <c r="B8" s="58" t="inlineStr">
         <is>
           <t>Q</t>
         </is>
       </c>
-      <c r="C8" s="27" t="inlineStr">
+      <c r="C8" s="44" t="inlineStr">
         <is>
           <t>Do I need to file Form 1040-ES?</t>
         </is>
@@ -3115,12 +4363,12 @@
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">
-      <c r="B11" s="35" t="inlineStr">
+      <c r="B11" s="58" t="inlineStr">
         <is>
           <t>Q</t>
         </is>
       </c>
-      <c r="C11" s="27" t="inlineStr">
+      <c r="C11" s="44" t="inlineStr">
         <is>
           <t>How does the state work?</t>
         </is>
@@ -3134,12 +4382,12 @@
       </c>
     </row>
     <row r="14" ht="22" customHeight="1">
-      <c r="B14" s="35" t="inlineStr">
+      <c r="B14" s="58" t="inlineStr">
         <is>
           <t>Q</t>
         </is>
       </c>
-      <c r="C14" s="27" t="inlineStr">
+      <c r="C14" s="44" t="inlineStr">
         <is>
           <t>What if my income is uneven across the year?</t>
         </is>
@@ -3153,12 +4401,12 @@
       </c>
     </row>
     <row r="17" ht="22" customHeight="1">
-      <c r="B17" s="35" t="inlineStr">
+      <c r="B17" s="58" t="inlineStr">
         <is>
           <t>Q</t>
         </is>
       </c>
-      <c r="C17" s="27" t="inlineStr">
+      <c r="C17" s="44" t="inlineStr">
         <is>
           <t>What's the actual penalty if I skip a quarter?</t>
         </is>
@@ -3172,12 +4420,12 @@
       </c>
     </row>
     <row r="20" ht="22" customHeight="1">
-      <c r="B20" s="35" t="inlineStr">
+      <c r="B20" s="58" t="inlineStr">
         <is>
           <t>Q</t>
         </is>
       </c>
-      <c r="C20" s="27" t="inlineStr">
+      <c r="C20" s="44" t="inlineStr">
         <is>
           <t>Can I overpay to be safe?</t>
         </is>
@@ -3191,12 +4439,12 @@
       </c>
     </row>
     <row r="23" ht="22" customHeight="1">
-      <c r="B23" s="35" t="inlineStr">
+      <c r="B23" s="58" t="inlineStr">
         <is>
           <t>Q</t>
         </is>
       </c>
-      <c r="C23" s="27" t="inlineStr">
+      <c r="C23" s="44" t="inlineStr">
         <is>
           <t>I had a huge year. Last year was tiny. Do I really only owe what last year's tax was × 4?</t>
         </is>
@@ -3210,12 +4458,12 @@
       </c>
     </row>
     <row r="26" ht="22" customHeight="1">
-      <c r="B26" s="35" t="inlineStr">
+      <c r="B26" s="58" t="inlineStr">
         <is>
           <t>Q</t>
         </is>
       </c>
-      <c r="C26" s="27" t="inlineStr">
+      <c r="C26" s="44" t="inlineStr">
         <is>
           <t>What if I miss a quarter and want to catch up?</t>
         </is>
@@ -3229,12 +4477,12 @@
       </c>
     </row>
     <row r="29" ht="22" customHeight="1">
-      <c r="B29" s="35" t="inlineStr">
+      <c r="B29" s="58" t="inlineStr">
         <is>
           <t>Q</t>
         </is>
       </c>
-      <c r="C29" s="27" t="inlineStr">
+      <c r="C29" s="44" t="inlineStr">
         <is>
           <t>Does this work if I'm both W-2 and self-employed?</t>
         </is>
@@ -3248,12 +4496,12 @@
       </c>
     </row>
     <row r="32" ht="22" customHeight="1">
-      <c r="B32" s="35" t="inlineStr">
+      <c r="B32" s="58" t="inlineStr">
         <is>
           <t>Q</t>
         </is>
       </c>
-      <c r="C32" s="27" t="inlineStr">
+      <c r="C32" s="44" t="inlineStr">
         <is>
           <t>Do I need to keep records of payments?</t>
         </is>

</xml_diff>

<commit_message>
fix: replace openpyxl bar chart with cell-based progress table on Dashboard
The openpyxl-generated BarChart was rendering with overlapping x-axis
labels in Numbers/Sheets (a known compatibility quirk where series titles
get concatenated with category labels).

Replaced with a native cell table: Quarter / Due / Target / Paid /
Remaining / % paid / Progress. The progress bar is a REPT("█",...) +
REPT("░",...) text formula that renders identically in Excel, Numbers,
and Google Sheets — no chart-object rendering bugs possible. Paid cells
get green/amber conditional fills based on payment status.
</commit_message>
<xml_diff>
--- a/products/quarterly-tax-system-2026.xlsx
+++ b/products/quarterly-tax-system-2026.xlsx
@@ -58,7 +58,7 @@
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0"/>
     <numFmt numFmtId="166" formatCode="yyyy-mm-dd"/>
   </numFmts>
-  <fonts count="19">
+  <fonts count="20">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -172,6 +172,12 @@
       <color rgb="FF1C2B4A"/>
       <sz val="16"/>
     </font>
+    <font>
+      <name val="Consolas"/>
+      <b val="1"/>
+      <color rgb="FFC9973A"/>
+      <sz val="11"/>
+    </font>
   </fonts>
   <fills count="8">
     <fill>
@@ -217,7 +223,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="18">
+  <borders count="21">
     <border>
       <left/>
       <right/>
@@ -419,11 +425,44 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FF1C2B4A"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF1C2B4A"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF1C2B4A"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF1C2B4A"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF1C2B4A"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF1C2B4A"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="59">
+  <cellXfs count="63">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -500,30 +539,50 @@
     <xf numFmtId="0" fontId="12" fillId="6" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="6" fillId="3" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="6" fillId="3" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="3" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="6" fillId="3" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="3" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
     <xf numFmtId="165" fontId="4" fillId="3" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
@@ -536,9 +595,6 @@
     <xf numFmtId="165" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="165" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
@@ -547,15 +603,11 @@
     </xf>
     <xf numFmtId="165" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="166" fontId="4" fillId="3" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="9" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
@@ -570,9 +622,6 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -585,7 +634,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="8">
+  <dxfs count="12">
     <dxf>
       <font>
         <name val="Calibri"/>
@@ -606,6 +655,62 @@
         <b val="1"/>
         <color rgb="FFA86C0A"/>
         <sz val="16"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFEF6E8"/>
+          <bgColor rgb="FFFEF6E8"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Calibri"/>
+        <b val="1"/>
+        <color rgb="FF276944"/>
+        <sz val="11"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFEAF5EF"/>
+          <bgColor rgb="FFEAF5EF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Calibri"/>
+        <b val="1"/>
+        <color rgb="FFA86C0A"/>
+        <sz val="11"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFEF6E8"/>
+          <bgColor rgb="FFFEF6E8"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Calibri"/>
+        <b val="1"/>
+        <color rgb="FF276944"/>
+        <sz val="12"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFEAF5EF"/>
+          <bgColor rgb="FFEAF5EF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Calibri"/>
+        <b val="1"/>
+        <color rgb="FFA86C0A"/>
+        <sz val="12"/>
       </font>
       <fill>
         <patternFill patternType="solid">
@@ -760,179 +865,6 @@
     </indexedColors>
   </colors>
 </styleSheet>
-</file>
-
-<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="11"/>
-  <chart>
-    <title>
-      <tx>
-        <rich>
-          <a:bodyPr/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr/>
-            </a:pPr>
-            <a:r>
-              <a:t>Federal — Target vs Paid by Quarter</a:t>
-            </a:r>
-          </a:p>
-        </rich>
-      </tx>
-    </title>
-    <plotArea>
-      <barChart>
-        <barDir val="col"/>
-        <grouping val="clustered"/>
-        <ser>
-          <idx val="0"/>
-          <order val="0"/>
-          <tx>
-            <strRef>
-              <f>'Dashboard'!C22</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:solidFill>
-              <a:srgbClr val="1C2B4A"/>
-            </a:solidFill>
-            <a:ln>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <numRef>
-              <f>'Dashboard'!$B$23:$B$26</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Dashboard'!$C$23:$C$26</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="1"/>
-          <order val="1"/>
-          <tx>
-            <strRef>
-              <f>'Dashboard'!D22</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:solidFill>
-              <a:srgbClr val="C9973A"/>
-            </a:solidFill>
-            <a:ln>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <numRef>
-              <f>'Dashboard'!$B$23:$B$26</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Dashboard'!$D$23:$D$26</f>
-            </numRef>
-          </val>
-        </ser>
-        <dLbls>
-          <showVal val="0"/>
-        </dLbls>
-        <gapWidth val="150"/>
-        <axId val="10"/>
-        <axId val="100"/>
-      </barChart>
-      <catAx>
-        <axId val="10"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <axPos val="l"/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>Quarter</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="100"/>
-        <lblOffset val="100"/>
-      </catAx>
-      <valAx>
-        <axId val="100"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <axPos val="l"/>
-        <majorGridlines/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>Dollars</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="10"/>
-      </valAx>
-    </plotArea>
-    <legend>
-      <legendPos val="r"/>
-    </legend>
-    <plotVisOnly val="1"/>
-    <dispBlanksAs val="gap"/>
-  </chart>
-</chartSpace>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <oneCellAnchor>
-    <from>
-      <col>5</col>
-      <colOff>0</colOff>
-      <row>21</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="6480000" cy="2880000"/>
-    <graphicFrame>
-      <nvGraphicFramePr>
-        <cNvPr id="1" name="Chart 1"/>
-        <cNvGraphicFramePr/>
-      </nvGraphicFramePr>
-      <xfrm/>
-      <a:graphic>
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
-        </a:graphicData>
-      </a:graphic>
-    </graphicFrame>
-    <clientData/>
-  </oneCellAnchor>
-</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1509,7 +1441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:J40"/>
+  <dimension ref="B2:J30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -1518,10 +1450,10 @@
     <col width="20" customWidth="1" min="4" max="4"/>
     <col width="20" customWidth="1" min="5" max="5"/>
     <col width="2" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
-    <col width="20" customWidth="1" min="8" max="8"/>
-    <col width="20" customWidth="1" min="9" max="9"/>
-    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="2" ht="36" customHeight="1">
@@ -1699,98 +1631,223 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="18" customHeight="1">
+    <row r="22" ht="26" customHeight="1">
       <c r="B22" s="30" t="inlineStr">
         <is>
           <t>Quarter</t>
         </is>
       </c>
-      <c r="C22" s="31" t="inlineStr">
+      <c r="C22" s="30" t="inlineStr">
+        <is>
+          <t>Due date</t>
+        </is>
+      </c>
+      <c r="D22" s="30" t="inlineStr">
         <is>
           <t>Target $</t>
         </is>
       </c>
-      <c r="D22" s="31" t="inlineStr">
+      <c r="E22" s="30" t="inlineStr">
         <is>
           <t>Paid $</t>
         </is>
       </c>
-    </row>
-    <row r="23" ht="18" customHeight="1">
-      <c r="B23" s="30" t="inlineStr">
+      <c r="G22" s="30" t="inlineStr">
+        <is>
+          <t>Remaining</t>
+        </is>
+      </c>
+      <c r="H22" s="30" t="inlineStr">
+        <is>
+          <t>% paid</t>
+        </is>
+      </c>
+      <c r="I22" s="30" t="inlineStr">
+        <is>
+          <t>Progress</t>
+        </is>
+      </c>
+      <c r="J22" s="31" t="n"/>
+    </row>
+    <row r="23" ht="26" customHeight="1">
+      <c r="B23" s="32" t="inlineStr">
         <is>
           <t>Q1</t>
         </is>
       </c>
-      <c r="C23" s="32">
+      <c r="C23" s="8" t="inlineStr">
+        <is>
+          <t>April 15</t>
+        </is>
+      </c>
+      <c r="D23" s="33">
         <f>'Quarterly Payments'!$D$7</f>
         <v/>
       </c>
-      <c r="D23" s="32">
+      <c r="E23" s="33">
         <f>'Quarterly Payments'!$F$7</f>
         <v/>
       </c>
-    </row>
-    <row r="24" ht="18" customHeight="1">
-      <c r="B24" s="30" t="inlineStr">
+      <c r="G23" s="33">
+        <f>MAX(D23-E23,0)</f>
+        <v/>
+      </c>
+      <c r="H23" s="34">
+        <f>IFERROR(E23/D23,0)</f>
+        <v/>
+      </c>
+      <c r="I23" s="35">
+        <f>IF(D23=0,REPT("░",20),REPT("█",MIN(20,ROUND(E23/D23*20,0)))&amp;REPT("░",MAX(0,20-ROUND(E23/D23*20,0))))</f>
+        <v/>
+      </c>
+      <c r="J23" s="11" t="n"/>
+    </row>
+    <row r="24" ht="26" customHeight="1">
+      <c r="B24" s="32" t="inlineStr">
         <is>
           <t>Q2</t>
         </is>
       </c>
-      <c r="C24" s="32">
+      <c r="C24" s="8" t="inlineStr">
+        <is>
+          <t>June 15</t>
+        </is>
+      </c>
+      <c r="D24" s="33">
         <f>'Quarterly Payments'!$D$8</f>
         <v/>
       </c>
-      <c r="D24" s="32">
+      <c r="E24" s="33">
         <f>'Quarterly Payments'!$F$8</f>
         <v/>
       </c>
-    </row>
-    <row r="25" ht="18" customHeight="1">
-      <c r="B25" s="30" t="inlineStr">
+      <c r="G24" s="33">
+        <f>MAX(D24-E24,0)</f>
+        <v/>
+      </c>
+      <c r="H24" s="34">
+        <f>IFERROR(E24/D24,0)</f>
+        <v/>
+      </c>
+      <c r="I24" s="35">
+        <f>IF(D24=0,REPT("░",20),REPT("█",MIN(20,ROUND(E24/D24*20,0)))&amp;REPT("░",MAX(0,20-ROUND(E24/D24*20,0))))</f>
+        <v/>
+      </c>
+      <c r="J24" s="11" t="n"/>
+    </row>
+    <row r="25" ht="26" customHeight="1">
+      <c r="B25" s="32" t="inlineStr">
         <is>
           <t>Q3</t>
         </is>
       </c>
-      <c r="C25" s="32">
+      <c r="C25" s="8" t="inlineStr">
+        <is>
+          <t>September 15</t>
+        </is>
+      </c>
+      <c r="D25" s="33">
         <f>'Quarterly Payments'!$D$9</f>
         <v/>
       </c>
-      <c r="D25" s="32">
+      <c r="E25" s="33">
         <f>'Quarterly Payments'!$F$9</f>
         <v/>
       </c>
-    </row>
-    <row r="26" ht="18" customHeight="1">
-      <c r="B26" s="30" t="inlineStr">
+      <c r="G25" s="33">
+        <f>MAX(D25-E25,0)</f>
+        <v/>
+      </c>
+      <c r="H25" s="34">
+        <f>IFERROR(E25/D25,0)</f>
+        <v/>
+      </c>
+      <c r="I25" s="35">
+        <f>IF(D25=0,REPT("░",20),REPT("█",MIN(20,ROUND(E25/D25*20,0)))&amp;REPT("░",MAX(0,20-ROUND(E25/D25*20,0))))</f>
+        <v/>
+      </c>
+      <c r="J25" s="11" t="n"/>
+    </row>
+    <row r="26" ht="26" customHeight="1">
+      <c r="B26" s="32" t="inlineStr">
         <is>
           <t>Q4</t>
         </is>
       </c>
-      <c r="C26" s="32">
+      <c r="C26" s="8" t="inlineStr">
+        <is>
+          <t>January 15</t>
+        </is>
+      </c>
+      <c r="D26" s="33">
         <f>'Quarterly Payments'!$D$10</f>
         <v/>
       </c>
-      <c r="D26" s="32">
+      <c r="E26" s="33">
         <f>'Quarterly Payments'!$F$10</f>
         <v/>
       </c>
-    </row>
-    <row r="40" ht="40" customHeight="1">
-      <c r="B40" s="33" t="inlineStr">
+      <c r="G26" s="33">
+        <f>MAX(D26-E26,0)</f>
+        <v/>
+      </c>
+      <c r="H26" s="34">
+        <f>IFERROR(E26/D26,0)</f>
+        <v/>
+      </c>
+      <c r="I26" s="35">
+        <f>IF(D26=0,REPT("░",20),REPT("█",MIN(20,ROUND(E26/D26*20,0)))&amp;REPT("░",MAX(0,20-ROUND(E26/D26*20,0))))</f>
+        <v/>
+      </c>
+      <c r="J26" s="11" t="n"/>
+    </row>
+    <row r="27" ht="30" customHeight="1">
+      <c r="B27" s="36" t="inlineStr">
+        <is>
+          <t>Annual total</t>
+        </is>
+      </c>
+      <c r="C27" s="37" t="n"/>
+      <c r="D27" s="38">
+        <f>SUM(D23:D26)</f>
+        <v/>
+      </c>
+      <c r="E27" s="38">
+        <f>SUM(E23:E26)</f>
+        <v/>
+      </c>
+      <c r="G27" s="38">
+        <f>MAX(D27-E27,0)</f>
+        <v/>
+      </c>
+      <c r="H27" s="39">
+        <f>IFERROR(E27/D27,0)</f>
+        <v/>
+      </c>
+      <c r="I27" s="40">
+        <f>IF(D27=0,REPT("░",20),REPT("█",MIN(20,ROUND(E27/D27*20,0)))&amp;REPT("░",MAX(0,20-ROUND(E27/D27*20,0))))</f>
+        <v/>
+      </c>
+      <c r="J27" s="37" t="n"/>
+    </row>
+    <row r="30" ht="40" customHeight="1">
+      <c r="B30" s="41" t="inlineStr">
         <is>
           <t>Everything on this Dashboard is calculated from the Setup, Income Forecast, and Quarterly Payments tabs. If a number looks wrong, the source is on those tabs — not here.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="27">
+  <mergeCells count="34">
     <mergeCell ref="G12:H12"/>
     <mergeCell ref="I6:J6"/>
     <mergeCell ref="B7:C7"/>
     <mergeCell ref="G11:H11"/>
     <mergeCell ref="I11:J11"/>
+    <mergeCell ref="I27:J27"/>
     <mergeCell ref="G16:J16"/>
+    <mergeCell ref="B27:C27"/>
+    <mergeCell ref="I26:J26"/>
     <mergeCell ref="B12:C12"/>
     <mergeCell ref="D6:E6"/>
     <mergeCell ref="G7:H7"/>
@@ -1798,15 +1855,19 @@
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="I7:J7"/>
     <mergeCell ref="D11:E11"/>
+    <mergeCell ref="I25:J25"/>
     <mergeCell ref="B16:E16"/>
-    <mergeCell ref="B40:J40"/>
     <mergeCell ref="G6:H6"/>
+    <mergeCell ref="I22:J22"/>
+    <mergeCell ref="B30:J30"/>
     <mergeCell ref="B15:J15"/>
     <mergeCell ref="I12:J12"/>
     <mergeCell ref="B5:J5"/>
     <mergeCell ref="D7:E7"/>
     <mergeCell ref="G17:J17"/>
     <mergeCell ref="B20:J20"/>
+    <mergeCell ref="I24:J24"/>
+    <mergeCell ref="I23:J23"/>
     <mergeCell ref="D12:E12"/>
     <mergeCell ref="B6:C6"/>
     <mergeCell ref="B17:E17"/>
@@ -1821,8 +1882,71 @@
       <formula>ISNUMBER(SEARCH("Not yet",B17))</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="E23">
+    <cfRule type="expression" priority="3" dxfId="2">
+      <formula>AND(E23&gt;=D23,D23&gt;0)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="4" dxfId="3">
+      <formula>AND(E23&gt;0,E23&lt;D23)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H23">
+    <cfRule type="expression" priority="5" dxfId="4">
+      <formula>H23&gt;=1</formula>
+    </cfRule>
+    <cfRule type="expression" priority="6" dxfId="5">
+      <formula>AND(H23&gt;0,H23&lt;1)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E24">
+    <cfRule type="expression" priority="7" dxfId="2">
+      <formula>AND(E24&gt;=D24,D24&gt;0)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="8" dxfId="3">
+      <formula>AND(E24&gt;0,E24&lt;D24)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H24">
+    <cfRule type="expression" priority="9" dxfId="4">
+      <formula>H24&gt;=1</formula>
+    </cfRule>
+    <cfRule type="expression" priority="10" dxfId="5">
+      <formula>AND(H24&gt;0,H24&lt;1)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E25">
+    <cfRule type="expression" priority="11" dxfId="2">
+      <formula>AND(E25&gt;=D25,D25&gt;0)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="12" dxfId="3">
+      <formula>AND(E25&gt;0,E25&lt;D25)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H25">
+    <cfRule type="expression" priority="13" dxfId="4">
+      <formula>H25&gt;=1</formula>
+    </cfRule>
+    <cfRule type="expression" priority="14" dxfId="5">
+      <formula>AND(H25&gt;0,H25&lt;1)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E26">
+    <cfRule type="expression" priority="15" dxfId="2">
+      <formula>AND(E26&gt;=D26,D26&gt;0)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="16" dxfId="3">
+      <formula>AND(E26&gt;0,E26&lt;D26)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H26">
+    <cfRule type="expression" priority="17" dxfId="4">
+      <formula>H26&gt;=1</formula>
+    </cfRule>
+    <cfRule type="expression" priority="18" dxfId="5">
+      <formula>AND(H26&gt;0,H26&lt;1)</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1842,7 +1966,7 @@
   </cols>
   <sheetData>
     <row r="2" ht="32" customHeight="1">
-      <c r="B2" s="34" t="inlineStr">
+      <c r="B2" s="42" t="inlineStr">
         <is>
           <t>Setup</t>
         </is>
@@ -1863,12 +1987,12 @@
       </c>
     </row>
     <row r="6" ht="24" customHeight="1">
-      <c r="B6" s="30" t="inlineStr">
+      <c r="B6" s="43" t="inlineStr">
         <is>
           <t>Tax year</t>
         </is>
       </c>
-      <c r="C6" s="35" t="n">
+      <c r="C6" s="44" t="n">
         <v>2026</v>
       </c>
       <c r="D6" s="15" t="inlineStr">
@@ -1878,12 +2002,12 @@
       </c>
     </row>
     <row r="7" ht="24" customHeight="1">
-      <c r="B7" s="30" t="inlineStr">
+      <c r="B7" s="43" t="inlineStr">
         <is>
           <t>Filing status</t>
         </is>
       </c>
-      <c r="C7" s="35" t="inlineStr">
+      <c r="C7" s="44" t="inlineStr">
         <is>
           <t>Single</t>
         </is>
@@ -1895,12 +2019,12 @@
       </c>
     </row>
     <row r="8" ht="24" customHeight="1">
-      <c r="B8" s="30" t="inlineStr">
+      <c r="B8" s="43" t="inlineStr">
         <is>
           <t>State</t>
         </is>
       </c>
-      <c r="C8" s="35" t="inlineStr">
+      <c r="C8" s="44" t="inlineStr">
         <is>
           <t>CA</t>
         </is>
@@ -1912,12 +2036,12 @@
       </c>
     </row>
     <row r="9" ht="24" customHeight="1">
-      <c r="B9" s="30" t="inlineStr">
+      <c r="B9" s="43" t="inlineStr">
         <is>
           <t>State flat estimated tax rate</t>
         </is>
       </c>
-      <c r="C9" s="36" t="n">
+      <c r="C9" s="45" t="n">
         <v>0.06</v>
       </c>
       <c r="D9" s="15" t="inlineStr">
@@ -1934,12 +2058,12 @@
       </c>
     </row>
     <row r="12" ht="24" customHeight="1">
-      <c r="B12" s="30" t="inlineStr">
+      <c r="B12" s="43" t="inlineStr">
         <is>
           <t>Estimated net self-employment income (annual)</t>
         </is>
       </c>
-      <c r="C12" s="37" t="n">
+      <c r="C12" s="38" t="n">
         <v>0</v>
       </c>
       <c r="D12" s="15" t="inlineStr">
@@ -1949,12 +2073,12 @@
       </c>
     </row>
     <row r="13" ht="24" customHeight="1">
-      <c r="B13" s="30" t="inlineStr">
+      <c r="B13" s="43" t="inlineStr">
         <is>
           <t>W-2 income (if you also have a day job)</t>
         </is>
       </c>
-      <c r="C13" s="37" t="n">
+      <c r="C13" s="38" t="n">
         <v>0</v>
       </c>
       <c r="D13" s="15" t="inlineStr">
@@ -1964,12 +2088,12 @@
       </c>
     </row>
     <row r="14" ht="24" customHeight="1">
-      <c r="B14" s="30" t="inlineStr">
+      <c r="B14" s="43" t="inlineStr">
         <is>
           <t>Federal tax withheld from W-2 (this year)</t>
         </is>
       </c>
-      <c r="C14" s="37" t="n">
+      <c r="C14" s="38" t="n">
         <v>0</v>
       </c>
       <c r="D14" s="15" t="inlineStr">
@@ -1986,12 +2110,12 @@
       </c>
     </row>
     <row r="17" ht="24" customHeight="1">
-      <c r="B17" s="30" t="inlineStr">
+      <c r="B17" s="43" t="inlineStr">
         <is>
           <t>Total federal tax owed last year (Form 1040 line 24)</t>
         </is>
       </c>
-      <c r="C17" s="37" t="n">
+      <c r="C17" s="38" t="n">
         <v>0</v>
       </c>
       <c r="D17" s="15" t="inlineStr">
@@ -2001,12 +2125,12 @@
       </c>
     </row>
     <row r="18" ht="24" customHeight="1">
-      <c r="B18" s="30" t="inlineStr">
+      <c r="B18" s="43" t="inlineStr">
         <is>
           <t>Last year's AGI (Form 1040 line 11)</t>
         </is>
       </c>
-      <c r="C18" s="37" t="n">
+      <c r="C18" s="38" t="n">
         <v>0</v>
       </c>
       <c r="D18" s="15" t="inlineStr">
@@ -2023,12 +2147,12 @@
       </c>
     </row>
     <row r="21" ht="24" customHeight="1">
-      <c r="B21" s="30" t="inlineStr">
+      <c r="B21" s="43" t="inlineStr">
         <is>
           <t>Standard deduction (single / MFS)</t>
         </is>
       </c>
-      <c r="C21" s="37" t="n">
+      <c r="C21" s="38" t="n">
         <v>15750</v>
       </c>
       <c r="D21" s="15" t="inlineStr">
@@ -2038,12 +2162,12 @@
       </c>
     </row>
     <row r="22" ht="24" customHeight="1">
-      <c r="B22" s="30" t="inlineStr">
+      <c r="B22" s="43" t="inlineStr">
         <is>
           <t>Standard deduction (MFJ)</t>
         </is>
       </c>
-      <c r="C22" s="37" t="n">
+      <c r="C22" s="38" t="n">
         <v>31500</v>
       </c>
       <c r="D22" s="15" t="inlineStr">
@@ -2053,12 +2177,12 @@
       </c>
     </row>
     <row r="23" ht="24" customHeight="1">
-      <c r="B23" s="30" t="inlineStr">
+      <c r="B23" s="43" t="inlineStr">
         <is>
           <t>Standard deduction (HOH)</t>
         </is>
       </c>
-      <c r="C23" s="37" t="n">
+      <c r="C23" s="38" t="n">
         <v>23625</v>
       </c>
       <c r="D23" s="15" t="inlineStr">
@@ -2068,12 +2192,12 @@
       </c>
     </row>
     <row r="24" ht="24" customHeight="1">
-      <c r="B24" s="30" t="inlineStr">
+      <c r="B24" s="43" t="inlineStr">
         <is>
           <t>Social Security wage base</t>
         </is>
       </c>
-      <c r="C24" s="37" t="n">
+      <c r="C24" s="38" t="n">
         <v>176100</v>
       </c>
       <c r="D24" s="15" t="inlineStr">
@@ -2107,84 +2231,84 @@
       </c>
     </row>
     <row r="28" ht="20" customHeight="1">
-      <c r="B28" s="38" t="n">
+      <c r="B28" s="46" t="n">
         <v>11925</v>
       </c>
-      <c r="C28" s="38" t="n">
+      <c r="C28" s="46" t="n">
         <v>23850</v>
       </c>
-      <c r="D28" s="39" t="n">
+      <c r="D28" s="47" t="n">
         <v>0.1</v>
       </c>
     </row>
     <row r="29" ht="20" customHeight="1">
-      <c r="B29" s="38" t="n">
+      <c r="B29" s="46" t="n">
         <v>48475</v>
       </c>
-      <c r="C29" s="38" t="n">
+      <c r="C29" s="46" t="n">
         <v>96950</v>
       </c>
-      <c r="D29" s="39" t="n">
+      <c r="D29" s="47" t="n">
         <v>0.12</v>
       </c>
     </row>
     <row r="30" ht="20" customHeight="1">
-      <c r="B30" s="38" t="n">
+      <c r="B30" s="46" t="n">
         <v>103350</v>
       </c>
-      <c r="C30" s="38" t="n">
+      <c r="C30" s="46" t="n">
         <v>206700</v>
       </c>
-      <c r="D30" s="39" t="n">
+      <c r="D30" s="47" t="n">
         <v>0.22</v>
       </c>
     </row>
     <row r="31" ht="20" customHeight="1">
-      <c r="B31" s="38" t="n">
+      <c r="B31" s="46" t="n">
         <v>197300</v>
       </c>
-      <c r="C31" s="38" t="n">
+      <c r="C31" s="46" t="n">
         <v>394600</v>
       </c>
-      <c r="D31" s="39" t="n">
+      <c r="D31" s="47" t="n">
         <v>0.24</v>
       </c>
     </row>
     <row r="32" ht="20" customHeight="1">
-      <c r="B32" s="38" t="n">
+      <c r="B32" s="46" t="n">
         <v>250525</v>
       </c>
-      <c r="C32" s="38" t="n">
+      <c r="C32" s="46" t="n">
         <v>501050</v>
       </c>
-      <c r="D32" s="39" t="n">
+      <c r="D32" s="47" t="n">
         <v>0.32</v>
       </c>
     </row>
     <row r="33" ht="20" customHeight="1">
-      <c r="B33" s="38" t="n">
+      <c r="B33" s="46" t="n">
         <v>626350</v>
       </c>
-      <c r="C33" s="38" t="n">
+      <c r="C33" s="46" t="n">
         <v>751600</v>
       </c>
-      <c r="D33" s="39" t="n">
+      <c r="D33" s="47" t="n">
         <v>0.35</v>
       </c>
     </row>
     <row r="34" ht="20" customHeight="1">
-      <c r="B34" s="38" t="n">
+      <c r="B34" s="46" t="n">
         <v>999999999</v>
       </c>
-      <c r="C34" s="38" t="n">
+      <c r="C34" s="46" t="n">
         <v>999999999</v>
       </c>
-      <c r="D34" s="39" t="n">
+      <c r="D34" s="47" t="n">
         <v>0.37</v>
       </c>
     </row>
     <row r="36" ht="36" customHeight="1">
-      <c r="B36" s="33" t="inlineStr">
+      <c r="B36" s="41" t="inlineStr">
         <is>
           <t>HoH and MFS brackets aren't modeled separately — if you use those statuses, set filing status above to the closest match (HOH → MFJ for brackets, MFS → Single) and adjust the standard deduction. For complex returns, consult a CPA.</t>
         </is>
@@ -2232,7 +2356,7 @@
   </cols>
   <sheetData>
     <row r="2" ht="32" customHeight="1">
-      <c r="B2" s="34" t="inlineStr">
+      <c r="B2" s="42" t="inlineStr">
         <is>
           <t>Income Forecast</t>
         </is>
@@ -2288,7 +2412,7 @@
           <t>Other</t>
         </is>
       </c>
-      <c r="I5" s="40" t="inlineStr">
+      <c r="I5" s="48" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
@@ -2300,25 +2424,25 @@
           <t>January</t>
         </is>
       </c>
-      <c r="C6" s="38" t="n">
-        <v>0</v>
-      </c>
-      <c r="D6" s="38" t="n">
-        <v>0</v>
-      </c>
-      <c r="E6" s="38" t="n">
-        <v>0</v>
-      </c>
-      <c r="F6" s="38" t="n">
-        <v>0</v>
-      </c>
-      <c r="G6" s="38" t="n">
-        <v>0</v>
-      </c>
-      <c r="H6" s="38" t="n">
-        <v>0</v>
-      </c>
-      <c r="I6" s="41">
+      <c r="C6" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" s="49">
         <f>SUM(C6:H6)</f>
         <v/>
       </c>
@@ -2329,25 +2453,25 @@
           <t>February</t>
         </is>
       </c>
-      <c r="C7" s="38" t="n">
-        <v>0</v>
-      </c>
-      <c r="D7" s="38" t="n">
-        <v>0</v>
-      </c>
-      <c r="E7" s="38" t="n">
-        <v>0</v>
-      </c>
-      <c r="F7" s="38" t="n">
-        <v>0</v>
-      </c>
-      <c r="G7" s="38" t="n">
-        <v>0</v>
-      </c>
-      <c r="H7" s="38" t="n">
-        <v>0</v>
-      </c>
-      <c r="I7" s="41">
+      <c r="C7" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" s="49">
         <f>SUM(C7:H7)</f>
         <v/>
       </c>
@@ -2358,25 +2482,25 @@
           <t>March</t>
         </is>
       </c>
-      <c r="C8" s="38" t="n">
-        <v>0</v>
-      </c>
-      <c r="D8" s="38" t="n">
-        <v>0</v>
-      </c>
-      <c r="E8" s="38" t="n">
-        <v>0</v>
-      </c>
-      <c r="F8" s="38" t="n">
-        <v>0</v>
-      </c>
-      <c r="G8" s="38" t="n">
-        <v>0</v>
-      </c>
-      <c r="H8" s="38" t="n">
-        <v>0</v>
-      </c>
-      <c r="I8" s="41">
+      <c r="C8" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" s="49">
         <f>SUM(C8:H8)</f>
         <v/>
       </c>
@@ -2387,25 +2511,25 @@
           <t>April</t>
         </is>
       </c>
-      <c r="C9" s="38" t="n">
-        <v>0</v>
-      </c>
-      <c r="D9" s="38" t="n">
-        <v>0</v>
-      </c>
-      <c r="E9" s="38" t="n">
-        <v>0</v>
-      </c>
-      <c r="F9" s="38" t="n">
-        <v>0</v>
-      </c>
-      <c r="G9" s="38" t="n">
-        <v>0</v>
-      </c>
-      <c r="H9" s="38" t="n">
-        <v>0</v>
-      </c>
-      <c r="I9" s="41">
+      <c r="C9" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" s="49">
         <f>SUM(C9:H9)</f>
         <v/>
       </c>
@@ -2416,25 +2540,25 @@
           <t>May</t>
         </is>
       </c>
-      <c r="C10" s="38" t="n">
-        <v>0</v>
-      </c>
-      <c r="D10" s="38" t="n">
-        <v>0</v>
-      </c>
-      <c r="E10" s="38" t="n">
-        <v>0</v>
-      </c>
-      <c r="F10" s="38" t="n">
-        <v>0</v>
-      </c>
-      <c r="G10" s="38" t="n">
-        <v>0</v>
-      </c>
-      <c r="H10" s="38" t="n">
-        <v>0</v>
-      </c>
-      <c r="I10" s="41">
+      <c r="C10" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" s="49">
         <f>SUM(C10:H10)</f>
         <v/>
       </c>
@@ -2445,25 +2569,25 @@
           <t>June</t>
         </is>
       </c>
-      <c r="C11" s="38" t="n">
-        <v>0</v>
-      </c>
-      <c r="D11" s="38" t="n">
-        <v>0</v>
-      </c>
-      <c r="E11" s="38" t="n">
-        <v>0</v>
-      </c>
-      <c r="F11" s="38" t="n">
-        <v>0</v>
-      </c>
-      <c r="G11" s="38" t="n">
-        <v>0</v>
-      </c>
-      <c r="H11" s="38" t="n">
-        <v>0</v>
-      </c>
-      <c r="I11" s="41">
+      <c r="C11" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" s="49">
         <f>SUM(C11:H11)</f>
         <v/>
       </c>
@@ -2474,25 +2598,25 @@
           <t>July</t>
         </is>
       </c>
-      <c r="C12" s="38" t="n">
-        <v>0</v>
-      </c>
-      <c r="D12" s="38" t="n">
-        <v>0</v>
-      </c>
-      <c r="E12" s="38" t="n">
-        <v>0</v>
-      </c>
-      <c r="F12" s="38" t="n">
-        <v>0</v>
-      </c>
-      <c r="G12" s="38" t="n">
-        <v>0</v>
-      </c>
-      <c r="H12" s="38" t="n">
-        <v>0</v>
-      </c>
-      <c r="I12" s="41">
+      <c r="C12" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="D12" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" s="49">
         <f>SUM(C12:H12)</f>
         <v/>
       </c>
@@ -2503,25 +2627,25 @@
           <t>August</t>
         </is>
       </c>
-      <c r="C13" s="38" t="n">
-        <v>0</v>
-      </c>
-      <c r="D13" s="38" t="n">
-        <v>0</v>
-      </c>
-      <c r="E13" s="38" t="n">
-        <v>0</v>
-      </c>
-      <c r="F13" s="38" t="n">
-        <v>0</v>
-      </c>
-      <c r="G13" s="38" t="n">
-        <v>0</v>
-      </c>
-      <c r="H13" s="38" t="n">
-        <v>0</v>
-      </c>
-      <c r="I13" s="41">
+      <c r="C13" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="D13" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="I13" s="49">
         <f>SUM(C13:H13)</f>
         <v/>
       </c>
@@ -2532,25 +2656,25 @@
           <t>September</t>
         </is>
       </c>
-      <c r="C14" s="38" t="n">
-        <v>0</v>
-      </c>
-      <c r="D14" s="38" t="n">
-        <v>0</v>
-      </c>
-      <c r="E14" s="38" t="n">
-        <v>0</v>
-      </c>
-      <c r="F14" s="38" t="n">
-        <v>0</v>
-      </c>
-      <c r="G14" s="38" t="n">
-        <v>0</v>
-      </c>
-      <c r="H14" s="38" t="n">
-        <v>0</v>
-      </c>
-      <c r="I14" s="41">
+      <c r="C14" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="D14" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="I14" s="49">
         <f>SUM(C14:H14)</f>
         <v/>
       </c>
@@ -2561,25 +2685,25 @@
           <t>October</t>
         </is>
       </c>
-      <c r="C15" s="38" t="n">
-        <v>0</v>
-      </c>
-      <c r="D15" s="38" t="n">
-        <v>0</v>
-      </c>
-      <c r="E15" s="38" t="n">
-        <v>0</v>
-      </c>
-      <c r="F15" s="38" t="n">
-        <v>0</v>
-      </c>
-      <c r="G15" s="38" t="n">
-        <v>0</v>
-      </c>
-      <c r="H15" s="38" t="n">
-        <v>0</v>
-      </c>
-      <c r="I15" s="41">
+      <c r="C15" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="D15" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" s="49">
         <f>SUM(C15:H15)</f>
         <v/>
       </c>
@@ -2590,25 +2714,25 @@
           <t>November</t>
         </is>
       </c>
-      <c r="C16" s="38" t="n">
-        <v>0</v>
-      </c>
-      <c r="D16" s="38" t="n">
-        <v>0</v>
-      </c>
-      <c r="E16" s="38" t="n">
-        <v>0</v>
-      </c>
-      <c r="F16" s="38" t="n">
-        <v>0</v>
-      </c>
-      <c r="G16" s="38" t="n">
-        <v>0</v>
-      </c>
-      <c r="H16" s="38" t="n">
-        <v>0</v>
-      </c>
-      <c r="I16" s="41">
+      <c r="C16" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="D16" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" s="49">
         <f>SUM(C16:H16)</f>
         <v/>
       </c>
@@ -2619,60 +2743,60 @@
           <t>December</t>
         </is>
       </c>
-      <c r="C17" s="38" t="n">
-        <v>0</v>
-      </c>
-      <c r="D17" s="38" t="n">
-        <v>0</v>
-      </c>
-      <c r="E17" s="38" t="n">
-        <v>0</v>
-      </c>
-      <c r="F17" s="38" t="n">
-        <v>0</v>
-      </c>
-      <c r="G17" s="38" t="n">
-        <v>0</v>
-      </c>
-      <c r="H17" s="38" t="n">
-        <v>0</v>
-      </c>
-      <c r="I17" s="41">
+      <c r="C17" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="D17" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="I17" s="49">
         <f>SUM(C17:H17)</f>
         <v/>
       </c>
     </row>
     <row r="18" ht="30" customHeight="1">
-      <c r="B18" s="42" t="inlineStr">
+      <c r="B18" s="36" t="inlineStr">
         <is>
           <t>Annual total</t>
         </is>
       </c>
-      <c r="C18" s="37">
+      <c r="C18" s="38">
         <f>SUM(C6:C17)</f>
         <v/>
       </c>
-      <c r="D18" s="37">
+      <c r="D18" s="38">
         <f>SUM(D6:D17)</f>
         <v/>
       </c>
-      <c r="E18" s="37">
+      <c r="E18" s="38">
         <f>SUM(E6:E17)</f>
         <v/>
       </c>
-      <c r="F18" s="37">
+      <c r="F18" s="38">
         <f>SUM(F6:F17)</f>
         <v/>
       </c>
-      <c r="G18" s="37">
+      <c r="G18" s="38">
         <f>SUM(G6:G17)</f>
         <v/>
       </c>
-      <c r="H18" s="37">
+      <c r="H18" s="38">
         <f>SUM(H6:H17)</f>
         <v/>
       </c>
-      <c r="I18" s="37">
+      <c r="I18" s="38">
         <f>SUM(I6:I17)</f>
         <v/>
       </c>
@@ -2712,7 +2836,7 @@
           <t>Jan–Mar</t>
         </is>
       </c>
-      <c r="D22" s="43">
+      <c r="D22" s="50">
         <f>SUM(I6:I8)</f>
         <v/>
       </c>
@@ -2728,7 +2852,7 @@
           <t>Apr–May</t>
         </is>
       </c>
-      <c r="D23" s="43">
+      <c r="D23" s="50">
         <f>SUM(I9:I10)</f>
         <v/>
       </c>
@@ -2744,7 +2868,7 @@
           <t>Jun–Aug</t>
         </is>
       </c>
-      <c r="D24" s="43">
+      <c r="D24" s="50">
         <f>SUM(I11:I13)</f>
         <v/>
       </c>
@@ -2760,7 +2884,7 @@
           <t>Sep–Dec</t>
         </is>
       </c>
-      <c r="D25" s="43">
+      <c r="D25" s="50">
         <f>SUM(I14:I17)</f>
         <v/>
       </c>
@@ -2792,7 +2916,7 @@
   </cols>
   <sheetData>
     <row r="2" ht="32" customHeight="1">
-      <c r="B2" s="34" t="inlineStr">
+      <c r="B2" s="42" t="inlineStr">
         <is>
           <t>Tax Calculator</t>
         </is>
@@ -2813,12 +2937,12 @@
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
-      <c r="B6" s="30" t="inlineStr">
+      <c r="B6" s="43" t="inlineStr">
         <is>
           <t>Net SE income (this year)</t>
         </is>
       </c>
-      <c r="C6" s="41">
+      <c r="C6" s="49">
         <f>IF(SEOverride&gt;0,SEOverride,AnnualSEForecast)</f>
         <v/>
       </c>
@@ -2829,12 +2953,12 @@
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
-      <c r="B7" s="30" t="inlineStr">
+      <c r="B7" s="43" t="inlineStr">
         <is>
           <t>× 92.35% (SE tax base)</t>
         </is>
       </c>
-      <c r="C7" s="41">
+      <c r="C7" s="49">
         <f>'Tax Calculator'!$C$6*0.9235</f>
         <v/>
       </c>
@@ -2845,12 +2969,12 @@
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
-      <c r="B8" s="30" t="inlineStr">
+      <c r="B8" s="43" t="inlineStr">
         <is>
           <t>Social Security portion of SE tax (12.4% up to wage base)</t>
         </is>
       </c>
-      <c r="C8" s="41">
+      <c r="C8" s="49">
         <f>MIN('Tax Calculator'!$C$7,SSWageBase)*0.124</f>
         <v/>
       </c>
@@ -2861,12 +2985,12 @@
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="B9" s="30" t="inlineStr">
+      <c r="B9" s="43" t="inlineStr">
         <is>
           <t>Medicare portion of SE tax (2.9%)</t>
         </is>
       </c>
-      <c r="C9" s="41">
+      <c r="C9" s="49">
         <f>'Tax Calculator'!$C$7*0.029</f>
         <v/>
       </c>
@@ -2877,12 +3001,12 @@
       </c>
     </row>
     <row r="10" ht="26" customHeight="1">
-      <c r="B10" s="44" t="inlineStr">
+      <c r="B10" s="51" t="inlineStr">
         <is>
           <t>Total SE tax</t>
         </is>
       </c>
-      <c r="C10" s="45">
+      <c r="C10" s="52">
         <f>'Tax Calculator'!$C$8+'Tax Calculator'!$C$9</f>
         <v/>
       </c>
@@ -2893,12 +3017,12 @@
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">
-      <c r="B11" s="30" t="inlineStr">
+      <c r="B11" s="43" t="inlineStr">
         <is>
           <t>Deductible half of SE tax</t>
         </is>
       </c>
-      <c r="C11" s="41">
+      <c r="C11" s="49">
         <f>'Tax Calculator'!$C$10/2</f>
         <v/>
       </c>
@@ -2916,12 +3040,12 @@
       </c>
     </row>
     <row r="14" ht="22" customHeight="1">
-      <c r="B14" s="30" t="inlineStr">
+      <c r="B14" s="43" t="inlineStr">
         <is>
           <t>AGI (W-2 + net SE − half SE tax)</t>
         </is>
       </c>
-      <c r="C14" s="41">
+      <c r="C14" s="49">
         <f>W2Income+'Tax Calculator'!$C$6-'Tax Calculator'!$C$11</f>
         <v/>
       </c>
@@ -2932,12 +3056,12 @@
       </c>
     </row>
     <row r="15" ht="22" customHeight="1">
-      <c r="B15" s="30" t="inlineStr">
+      <c r="B15" s="43" t="inlineStr">
         <is>
           <t>Standard deduction (based on filing status)</t>
         </is>
       </c>
-      <c r="C15" s="41">
+      <c r="C15" s="49">
         <f>IF(FilingStatus="MFJ",StdDedMFJ,IF(FilingStatus="HOH",StdDedHOH,StdDedSingle))</f>
         <v/>
       </c>
@@ -2948,12 +3072,12 @@
       </c>
     </row>
     <row r="16" ht="22" customHeight="1">
-      <c r="B16" s="30" t="inlineStr">
+      <c r="B16" s="43" t="inlineStr">
         <is>
           <t>Taxable income</t>
         </is>
       </c>
-      <c r="C16" s="41">
+      <c r="C16" s="49">
         <f>MAX('Tax Calculator'!$C$14-'Tax Calculator'!$C$15,0)</f>
         <v/>
       </c>
@@ -2964,12 +3088,12 @@
       </c>
     </row>
     <row r="17" ht="26" customHeight="1">
-      <c r="B17" s="44" t="inlineStr">
+      <c r="B17" s="51" t="inlineStr">
         <is>
           <t>Federal income tax (bracket calc)</t>
         </is>
       </c>
-      <c r="C17" s="45">
+      <c r="C17" s="52">
         <f>IF(FilingStatus="MFJ",SUMPRODUCT(((MIN('Tax Calculator'!$C$16,BracketsMFJ)-IFERROR(OFFSET(BracketsMFJ,-1,0),0))&gt;0)*(MIN('Tax Calculator'!$C$16,BracketsMFJ)-IFERROR(OFFSET(BracketsMFJ,-1,0),0))*BracketsRate),SUMPRODUCT(((MIN('Tax Calculator'!$C$16,BracketsSingle)-IFERROR(OFFSET(BracketsSingle,-1,0),0))&gt;0)*(MIN('Tax Calculator'!$C$16,BracketsSingle)-IFERROR(OFFSET(BracketsSingle,-1,0),0))*BracketsRate))</f>
         <v/>
       </c>
@@ -2987,12 +3111,12 @@
       </c>
     </row>
     <row r="20" ht="26" customHeight="1">
-      <c r="B20" s="44" t="inlineStr">
+      <c r="B20" s="51" t="inlineStr">
         <is>
           <t>State income tax (flat rate × taxable income)</t>
         </is>
       </c>
-      <c r="C20" s="45">
+      <c r="C20" s="52">
         <f>'Tax Calculator'!$C$16*StateRate</f>
         <v/>
       </c>
@@ -3003,12 +3127,12 @@
       </c>
     </row>
     <row r="21" ht="22" customHeight="1">
-      <c r="B21" s="30" t="inlineStr">
+      <c r="B21" s="43" t="inlineStr">
         <is>
           <t>Total federal owed (SE + income)</t>
         </is>
       </c>
-      <c r="C21" s="41">
+      <c r="C21" s="49">
         <f>'Tax Calculator'!$C$10+'Tax Calculator'!$C$17</f>
         <v/>
       </c>
@@ -3019,12 +3143,12 @@
       </c>
     </row>
     <row r="22" ht="22" customHeight="1">
-      <c r="B22" s="30" t="inlineStr">
+      <c r="B22" s="43" t="inlineStr">
         <is>
           <t>Less: W-2 federal withholding</t>
         </is>
       </c>
-      <c r="C22" s="41">
+      <c r="C22" s="49">
         <f>-W2Withheld</f>
         <v/>
       </c>
@@ -3035,11 +3159,11 @@
       </c>
     </row>
     <row r="23" ht="26" customHeight="1">
-      <c r="B23" s="44">
+      <c r="B23" s="51">
         <f> Net federal owed (quarterly target)</f>
         <v/>
       </c>
-      <c r="C23" s="45">
+      <c r="C23" s="52">
         <f>'Tax Calculator'!$C$21-W2Withheld</f>
         <v/>
       </c>
@@ -3050,12 +3174,12 @@
       </c>
     </row>
     <row r="24" ht="26" customHeight="1">
-      <c r="B24" s="44" t="inlineStr">
+      <c r="B24" s="51" t="inlineStr">
         <is>
           <t>Total state owed (quarterly target)</t>
         </is>
       </c>
-      <c r="C24" s="45">
+      <c r="C24" s="52">
         <f>'Tax Calculator'!$C$20</f>
         <v/>
       </c>
@@ -3097,7 +3221,7 @@
   </cols>
   <sheetData>
     <row r="2" ht="32" customHeight="1">
-      <c r="B2" s="34" t="inlineStr">
+      <c r="B2" s="42" t="inlineStr">
         <is>
           <t>Quarterly Payments</t>
         </is>
@@ -3118,37 +3242,37 @@
       </c>
     </row>
     <row r="6" ht="24" customHeight="1">
-      <c r="B6" s="46" t="inlineStr">
+      <c r="B6" s="30" t="inlineStr">
         <is>
           <t>Q</t>
         </is>
       </c>
-      <c r="C6" s="46" t="inlineStr">
+      <c r="C6" s="30" t="inlineStr">
         <is>
           <t>Due date</t>
         </is>
       </c>
-      <c r="D6" s="46" t="inlineStr">
+      <c r="D6" s="30" t="inlineStr">
         <is>
           <t>Target $</t>
         </is>
       </c>
-      <c r="E6" s="46" t="inlineStr">
+      <c r="E6" s="30" t="inlineStr">
         <is>
           <t>Paid date</t>
         </is>
       </c>
-      <c r="F6" s="46" t="inlineStr">
+      <c r="F6" s="30" t="inlineStr">
         <is>
           <t>Paid $</t>
         </is>
       </c>
-      <c r="G6" s="46" t="inlineStr">
+      <c r="G6" s="30" t="inlineStr">
         <is>
           <t>Method</t>
         </is>
       </c>
-      <c r="H6" s="46" t="inlineStr">
+      <c r="H6" s="30" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
@@ -3165,13 +3289,13 @@
           <t>April 15</t>
         </is>
       </c>
-      <c r="D7" s="41">
+      <c r="D7" s="49">
         <f>NetFedOwed/4</f>
         <v/>
       </c>
-      <c r="E7" s="47" t="n"/>
-      <c r="F7" s="38" t="n"/>
-      <c r="G7" s="48" t="n"/>
+      <c r="E7" s="53" t="n"/>
+      <c r="F7" s="46" t="n"/>
+      <c r="G7" s="54" t="n"/>
       <c r="H7" s="10">
         <f>IF(F7="","Not paid yet",IF(F7&gt;=D7*0.95,"On track","Underpaid by $"&amp;TEXT(D7-F7,"#,##0")))</f>
         <v/>
@@ -3188,13 +3312,13 @@
           <t>June 15</t>
         </is>
       </c>
-      <c r="D8" s="41">
+      <c r="D8" s="49">
         <f>NetFedOwed/4</f>
         <v/>
       </c>
-      <c r="E8" s="47" t="n"/>
-      <c r="F8" s="38" t="n"/>
-      <c r="G8" s="48" t="n"/>
+      <c r="E8" s="53" t="n"/>
+      <c r="F8" s="46" t="n"/>
+      <c r="G8" s="54" t="n"/>
       <c r="H8" s="10">
         <f>IF(F8="","Not paid yet",IF(F8&gt;=D8*0.95,"On track","Underpaid by $"&amp;TEXT(D8-F8,"#,##0")))</f>
         <v/>
@@ -3211,13 +3335,13 @@
           <t>September 15</t>
         </is>
       </c>
-      <c r="D9" s="41">
+      <c r="D9" s="49">
         <f>NetFedOwed/4</f>
         <v/>
       </c>
-      <c r="E9" s="47" t="n"/>
-      <c r="F9" s="38" t="n"/>
-      <c r="G9" s="48" t="n"/>
+      <c r="E9" s="53" t="n"/>
+      <c r="F9" s="46" t="n"/>
+      <c r="G9" s="54" t="n"/>
       <c r="H9" s="10">
         <f>IF(F9="","Not paid yet",IF(F9&gt;=D9*0.95,"On track","Underpaid by $"&amp;TEXT(D9-F9,"#,##0")))</f>
         <v/>
@@ -3234,34 +3358,34 @@
           <t>January 15</t>
         </is>
       </c>
-      <c r="D10" s="41">
+      <c r="D10" s="49">
         <f>NetFedOwed/4</f>
         <v/>
       </c>
-      <c r="E10" s="47" t="n"/>
-      <c r="F10" s="38" t="n"/>
-      <c r="G10" s="48" t="n"/>
+      <c r="E10" s="53" t="n"/>
+      <c r="F10" s="46" t="n"/>
+      <c r="G10" s="54" t="n"/>
       <c r="H10" s="10">
         <f>IF(F10="","Not paid yet",IF(F10&gt;=D10*0.95,"On track","Underpaid by $"&amp;TEXT(D10-F10,"#,##0")))</f>
         <v/>
       </c>
     </row>
     <row r="11" ht="28" customHeight="1">
-      <c r="B11" s="42" t="inlineStr">
+      <c r="B11" s="36" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="C11" s="49" t="n"/>
-      <c r="D11" s="37">
+      <c r="C11" s="37" t="n"/>
+      <c r="D11" s="38">
         <f>SUM(D7:D10)</f>
         <v/>
       </c>
-      <c r="F11" s="37">
+      <c r="F11" s="38">
         <f>SUM(F7:F10)</f>
         <v/>
       </c>
-      <c r="H11" s="42">
+      <c r="H11" s="36">
         <f>IF(F11&gt;=D11*0.95,"Annual target met","Short $"&amp;TEXT(D11-F11,"#,##0"))</f>
         <v/>
       </c>
@@ -3274,37 +3398,37 @@
       </c>
     </row>
     <row r="15" ht="24" customHeight="1">
-      <c r="B15" s="46" t="inlineStr">
+      <c r="B15" s="30" t="inlineStr">
         <is>
           <t>Q</t>
         </is>
       </c>
-      <c r="C15" s="46" t="inlineStr">
+      <c r="C15" s="30" t="inlineStr">
         <is>
           <t>Due date</t>
         </is>
       </c>
-      <c r="D15" s="46" t="inlineStr">
+      <c r="D15" s="30" t="inlineStr">
         <is>
           <t>Target $</t>
         </is>
       </c>
-      <c r="E15" s="46" t="inlineStr">
+      <c r="E15" s="30" t="inlineStr">
         <is>
           <t>Paid date</t>
         </is>
       </c>
-      <c r="F15" s="46" t="inlineStr">
+      <c r="F15" s="30" t="inlineStr">
         <is>
           <t>Paid $</t>
         </is>
       </c>
-      <c r="G15" s="46" t="inlineStr">
+      <c r="G15" s="30" t="inlineStr">
         <is>
           <t>Method</t>
         </is>
       </c>
-      <c r="H15" s="46" t="inlineStr">
+      <c r="H15" s="30" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
@@ -3321,13 +3445,13 @@
           <t>April 15</t>
         </is>
       </c>
-      <c r="D16" s="41">
+      <c r="D16" s="49">
         <f>NetStateOwed/4</f>
         <v/>
       </c>
-      <c r="E16" s="47" t="n"/>
-      <c r="F16" s="38" t="n"/>
-      <c r="G16" s="48" t="n"/>
+      <c r="E16" s="53" t="n"/>
+      <c r="F16" s="46" t="n"/>
+      <c r="G16" s="54" t="n"/>
       <c r="H16" s="10">
         <f>IF(F16="","Not paid yet",IF(F16&gt;=D16*0.95,"On track","Underpaid by $"&amp;TEXT(D16-F16,"#,##0")))</f>
         <v/>
@@ -3344,13 +3468,13 @@
           <t>June 15</t>
         </is>
       </c>
-      <c r="D17" s="41">
+      <c r="D17" s="49">
         <f>NetStateOwed/4</f>
         <v/>
       </c>
-      <c r="E17" s="47" t="n"/>
-      <c r="F17" s="38" t="n"/>
-      <c r="G17" s="48" t="n"/>
+      <c r="E17" s="53" t="n"/>
+      <c r="F17" s="46" t="n"/>
+      <c r="G17" s="54" t="n"/>
       <c r="H17" s="10">
         <f>IF(F17="","Not paid yet",IF(F17&gt;=D17*0.95,"On track","Underpaid by $"&amp;TEXT(D17-F17,"#,##0")))</f>
         <v/>
@@ -3367,13 +3491,13 @@
           <t>September 15</t>
         </is>
       </c>
-      <c r="D18" s="41">
+      <c r="D18" s="49">
         <f>NetStateOwed/4</f>
         <v/>
       </c>
-      <c r="E18" s="47" t="n"/>
-      <c r="F18" s="38" t="n"/>
-      <c r="G18" s="48" t="n"/>
+      <c r="E18" s="53" t="n"/>
+      <c r="F18" s="46" t="n"/>
+      <c r="G18" s="54" t="n"/>
       <c r="H18" s="10">
         <f>IF(F18="","Not paid yet",IF(F18&gt;=D18*0.95,"On track","Underpaid by $"&amp;TEXT(D18-F18,"#,##0")))</f>
         <v/>
@@ -3390,30 +3514,30 @@
           <t>January 15</t>
         </is>
       </c>
-      <c r="D19" s="41">
+      <c r="D19" s="49">
         <f>NetStateOwed/4</f>
         <v/>
       </c>
-      <c r="E19" s="47" t="n"/>
-      <c r="F19" s="38" t="n"/>
-      <c r="G19" s="48" t="n"/>
+      <c r="E19" s="53" t="n"/>
+      <c r="F19" s="46" t="n"/>
+      <c r="G19" s="54" t="n"/>
       <c r="H19" s="10">
         <f>IF(F19="","Not paid yet",IF(F19&gt;=D19*0.95,"On track","Underpaid by $"&amp;TEXT(D19-F19,"#,##0")))</f>
         <v/>
       </c>
     </row>
     <row r="20" ht="28" customHeight="1">
-      <c r="B20" s="42" t="inlineStr">
+      <c r="B20" s="36" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="C20" s="49" t="n"/>
-      <c r="D20" s="37">
+      <c r="C20" s="37" t="n"/>
+      <c r="D20" s="38">
         <f>SUM(D16:D19)</f>
         <v/>
       </c>
-      <c r="F20" s="37">
+      <c r="F20" s="38">
         <f>SUM(F16:F19)</f>
         <v/>
       </c>
@@ -3428,98 +3552,98 @@
     <mergeCell ref="B5:H5"/>
   </mergeCells>
   <conditionalFormatting sqref="H7">
-    <cfRule type="expression" priority="1" dxfId="2">
+    <cfRule type="expression" priority="1" dxfId="6">
       <formula>ISNUMBER(SEARCH("On track",H7))</formula>
     </cfRule>
-    <cfRule type="expression" priority="2" dxfId="3">
+    <cfRule type="expression" priority="2" dxfId="7">
       <formula>ISNUMBER(SEARCH("Not paid",H7))</formula>
     </cfRule>
-    <cfRule type="expression" priority="3" dxfId="4">
+    <cfRule type="expression" priority="3" dxfId="8">
       <formula>ISNUMBER(SEARCH("Underpaid",H7))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H8">
-    <cfRule type="expression" priority="4" dxfId="2">
+    <cfRule type="expression" priority="4" dxfId="6">
       <formula>ISNUMBER(SEARCH("On track",H8))</formula>
     </cfRule>
-    <cfRule type="expression" priority="5" dxfId="3">
+    <cfRule type="expression" priority="5" dxfId="7">
       <formula>ISNUMBER(SEARCH("Not paid",H8))</formula>
     </cfRule>
-    <cfRule type="expression" priority="6" dxfId="4">
+    <cfRule type="expression" priority="6" dxfId="8">
       <formula>ISNUMBER(SEARCH("Underpaid",H8))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H9">
-    <cfRule type="expression" priority="7" dxfId="2">
+    <cfRule type="expression" priority="7" dxfId="6">
       <formula>ISNUMBER(SEARCH("On track",H9))</formula>
     </cfRule>
-    <cfRule type="expression" priority="8" dxfId="3">
+    <cfRule type="expression" priority="8" dxfId="7">
       <formula>ISNUMBER(SEARCH("Not paid",H9))</formula>
     </cfRule>
-    <cfRule type="expression" priority="9" dxfId="4">
+    <cfRule type="expression" priority="9" dxfId="8">
       <formula>ISNUMBER(SEARCH("Underpaid",H9))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H10">
-    <cfRule type="expression" priority="10" dxfId="2">
+    <cfRule type="expression" priority="10" dxfId="6">
       <formula>ISNUMBER(SEARCH("On track",H10))</formula>
     </cfRule>
-    <cfRule type="expression" priority="11" dxfId="3">
+    <cfRule type="expression" priority="11" dxfId="7">
       <formula>ISNUMBER(SEARCH("Not paid",H10))</formula>
     </cfRule>
-    <cfRule type="expression" priority="12" dxfId="4">
+    <cfRule type="expression" priority="12" dxfId="8">
       <formula>ISNUMBER(SEARCH("Underpaid",H10))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H11">
-    <cfRule type="expression" priority="13" dxfId="2">
+    <cfRule type="expression" priority="13" dxfId="6">
       <formula>ISNUMBER(SEARCH("met",H11))</formula>
     </cfRule>
-    <cfRule type="expression" priority="14" dxfId="4">
+    <cfRule type="expression" priority="14" dxfId="8">
       <formula>ISNUMBER(SEARCH("Short",H11))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H16">
-    <cfRule type="expression" priority="15" dxfId="2">
+    <cfRule type="expression" priority="15" dxfId="6">
       <formula>ISNUMBER(SEARCH("On track",H16))</formula>
     </cfRule>
-    <cfRule type="expression" priority="16" dxfId="3">
+    <cfRule type="expression" priority="16" dxfId="7">
       <formula>ISNUMBER(SEARCH("Not paid",H16))</formula>
     </cfRule>
-    <cfRule type="expression" priority="17" dxfId="4">
+    <cfRule type="expression" priority="17" dxfId="8">
       <formula>ISNUMBER(SEARCH("Underpaid",H16))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H17">
-    <cfRule type="expression" priority="18" dxfId="2">
+    <cfRule type="expression" priority="18" dxfId="6">
       <formula>ISNUMBER(SEARCH("On track",H17))</formula>
     </cfRule>
-    <cfRule type="expression" priority="19" dxfId="3">
+    <cfRule type="expression" priority="19" dxfId="7">
       <formula>ISNUMBER(SEARCH("Not paid",H17))</formula>
     </cfRule>
-    <cfRule type="expression" priority="20" dxfId="4">
+    <cfRule type="expression" priority="20" dxfId="8">
       <formula>ISNUMBER(SEARCH("Underpaid",H17))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H18">
-    <cfRule type="expression" priority="21" dxfId="2">
+    <cfRule type="expression" priority="21" dxfId="6">
       <formula>ISNUMBER(SEARCH("On track",H18))</formula>
     </cfRule>
-    <cfRule type="expression" priority="22" dxfId="3">
+    <cfRule type="expression" priority="22" dxfId="7">
       <formula>ISNUMBER(SEARCH("Not paid",H18))</formula>
     </cfRule>
-    <cfRule type="expression" priority="23" dxfId="4">
+    <cfRule type="expression" priority="23" dxfId="8">
       <formula>ISNUMBER(SEARCH("Underpaid",H18))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H19">
-    <cfRule type="expression" priority="24" dxfId="2">
+    <cfRule type="expression" priority="24" dxfId="6">
       <formula>ISNUMBER(SEARCH("On track",H19))</formula>
     </cfRule>
-    <cfRule type="expression" priority="25" dxfId="3">
+    <cfRule type="expression" priority="25" dxfId="7">
       <formula>ISNUMBER(SEARCH("Not paid",H19))</formula>
     </cfRule>
-    <cfRule type="expression" priority="26" dxfId="4">
+    <cfRule type="expression" priority="26" dxfId="8">
       <formula>ISNUMBER(SEARCH("Underpaid",H19))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3543,7 +3667,7 @@
   </cols>
   <sheetData>
     <row r="2" ht="32" customHeight="1">
-      <c r="B2" s="34" t="inlineStr">
+      <c r="B2" s="42" t="inlineStr">
         <is>
           <t>Safe Harbor Check</t>
         </is>
@@ -3564,12 +3688,12 @@
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
-      <c r="B6" s="30" t="inlineStr">
+      <c r="B6" s="43" t="inlineStr">
         <is>
           <t>Required multiplier (110% if last year AGI &gt; $150K, else 100%)</t>
         </is>
       </c>
-      <c r="C6" s="50">
+      <c r="C6" s="55">
         <f>IF(LastYearAGI&gt;150000,1.1,1)</f>
         <v/>
       </c>
@@ -3580,12 +3704,12 @@
       </c>
     </row>
     <row r="7" ht="26" customHeight="1">
-      <c r="B7" s="44" t="inlineStr">
+      <c r="B7" s="51" t="inlineStr">
         <is>
           <t>Safe harbor target (last year's tax × multiplier)</t>
         </is>
       </c>
-      <c r="C7" s="37">
+      <c r="C7" s="38">
         <f>LastYearTax*C6</f>
         <v/>
       </c>
@@ -3596,12 +3720,12 @@
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
-      <c r="B8" s="30" t="inlineStr">
+      <c r="B8" s="43" t="inlineStr">
         <is>
           <t>Paid so far (Q1–Q4 federal + W-2 withholding)</t>
         </is>
       </c>
-      <c r="C8" s="41">
+      <c r="C8" s="49">
         <f>FedPaidYTD+W2Withheld</f>
         <v/>
       </c>
@@ -3612,12 +3736,12 @@
       </c>
     </row>
     <row r="9" ht="32" customHeight="1">
-      <c r="B9" s="44" t="inlineStr">
+      <c r="B9" s="51" t="inlineStr">
         <is>
           <t>Safe Harbor 1 status:</t>
         </is>
       </c>
-      <c r="C9" s="51">
+      <c r="C9" s="56">
         <f>IF(C8&gt;=C7,"✓ SAFE","Short $"&amp;TEXT(C7-C8,"#,##0"))</f>
         <v/>
       </c>
@@ -3630,12 +3754,12 @@
       </c>
     </row>
     <row r="12" ht="22" customHeight="1">
-      <c r="B12" s="30" t="inlineStr">
+      <c r="B12" s="43" t="inlineStr">
         <is>
           <t>This year's projected total federal tax</t>
         </is>
       </c>
-      <c r="C12" s="41">
+      <c r="C12" s="49">
         <f>TotalFedTax</f>
         <v/>
       </c>
@@ -3646,12 +3770,12 @@
       </c>
     </row>
     <row r="13" ht="26" customHeight="1">
-      <c r="B13" s="44" t="inlineStr">
+      <c r="B13" s="51" t="inlineStr">
         <is>
           <t>Safe harbor target (90% of this year's tax)</t>
         </is>
       </c>
-      <c r="C13" s="37">
+      <c r="C13" s="38">
         <f>C12*0.9</f>
         <v/>
       </c>
@@ -3662,12 +3786,12 @@
       </c>
     </row>
     <row r="14" ht="22" customHeight="1">
-      <c r="B14" s="30" t="inlineStr">
+      <c r="B14" s="43" t="inlineStr">
         <is>
           <t>Paid so far (Q1–Q4 federal + W-2 withholding)</t>
         </is>
       </c>
-      <c r="C14" s="41">
+      <c r="C14" s="49">
         <f>FedPaidYTD+W2Withheld</f>
         <v/>
       </c>
@@ -3678,12 +3802,12 @@
       </c>
     </row>
     <row r="15" ht="32" customHeight="1">
-      <c r="B15" s="44" t="inlineStr">
+      <c r="B15" s="51" t="inlineStr">
         <is>
           <t>Safe Harbor 2 status:</t>
         </is>
       </c>
-      <c r="C15" s="51">
+      <c r="C15" s="56">
         <f>IF(C14&gt;=C13,"✓ SAFE","Short $"&amp;TEXT(C13-C14,"#,##0"))</f>
         <v/>
       </c>
@@ -3696,12 +3820,12 @@
       </c>
     </row>
     <row r="18" ht="38" customHeight="1">
-      <c r="B18" s="44" t="inlineStr">
+      <c r="B18" s="51" t="inlineStr">
         <is>
           <t>Overall status:</t>
         </is>
       </c>
-      <c r="C18" s="51">
+      <c r="C18" s="56">
         <f>IF(OR(C8&gt;=C7,C14&gt;=C13),"✓ YES — you're safe from penalty","⚠ Not yet — close one of the gaps above")</f>
         <v/>
       </c>
@@ -3723,26 +3847,26 @@
     <mergeCell ref="B20:D20"/>
   </mergeCells>
   <conditionalFormatting sqref="C9">
-    <cfRule type="expression" priority="1" dxfId="5">
+    <cfRule type="expression" priority="1" dxfId="9">
       <formula>ISNUMBER(SEARCH("SAFE",C9))</formula>
     </cfRule>
-    <cfRule type="expression" priority="2" dxfId="6">
+    <cfRule type="expression" priority="2" dxfId="10">
       <formula>ISNUMBER(SEARCH("Short",C9))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C15">
-    <cfRule type="expression" priority="3" dxfId="5">
+    <cfRule type="expression" priority="3" dxfId="9">
       <formula>ISNUMBER(SEARCH("SAFE",C15))</formula>
     </cfRule>
-    <cfRule type="expression" priority="4" dxfId="6">
+    <cfRule type="expression" priority="4" dxfId="10">
       <formula>ISNUMBER(SEARCH("Short",C15))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C18">
-    <cfRule type="expression" priority="5" dxfId="5">
+    <cfRule type="expression" priority="5" dxfId="9">
       <formula>ISNUMBER(SEARCH("YES",C18))</formula>
     </cfRule>
-    <cfRule type="expression" priority="6" dxfId="7">
+    <cfRule type="expression" priority="6" dxfId="11">
       <formula>ISNUMBER(SEARCH("Not yet",C18))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3767,7 +3891,7 @@
   </cols>
   <sheetData>
     <row r="2" ht="32" customHeight="1">
-      <c r="B2" s="34" t="inlineStr">
+      <c r="B2" s="42" t="inlineStr">
         <is>
           <t>Worked Examples</t>
         </is>
@@ -3781,7 +3905,7 @@
       </c>
     </row>
     <row r="5" ht="28" customHeight="1">
-      <c r="B5" s="52" t="inlineStr"/>
+      <c r="B5" s="57" t="inlineStr"/>
       <c r="C5" s="7" t="inlineStr">
         <is>
           <t>DoorDash full-timer</t>
@@ -3804,17 +3928,17 @@
           <t>Situation</t>
         </is>
       </c>
-      <c r="C6" s="53" t="inlineStr">
+      <c r="C6" s="58" t="inlineStr">
         <is>
           <t>Single, lives in CA, Dashes full time. Tracked 22,000 business miles. Gross earnings $58,000 minus $15,400 mileage deduction = $42,600 net.</t>
         </is>
       </c>
-      <c r="D6" s="53" t="inlineStr">
+      <c r="D6" s="58" t="inlineStr">
         <is>
           <t>MFJ, NY, $48K W-2 day job with $5,400 federal withholding + $60K net freelance design work on the side.</t>
         </is>
       </c>
-      <c r="E6" s="53" t="inlineStr">
+      <c r="E6" s="58" t="inlineStr">
         <is>
           <t>Single, TX (no state tax), Etsy print shop. $25,000 net profit after COGS and home office deduction.</t>
         </is>
@@ -3833,17 +3957,17 @@
           <t>Filing status</t>
         </is>
       </c>
-      <c r="C9" s="54" t="inlineStr">
+      <c r="C9" s="59" t="inlineStr">
         <is>
           <t>Single</t>
         </is>
       </c>
-      <c r="D9" s="54" t="inlineStr">
+      <c r="D9" s="59" t="inlineStr">
         <is>
           <t>MFJ</t>
         </is>
       </c>
-      <c r="E9" s="54" t="inlineStr">
+      <c r="E9" s="59" t="inlineStr">
         <is>
           <t>Single</t>
         </is>
@@ -3855,17 +3979,17 @@
           <t>State</t>
         </is>
       </c>
-      <c r="C10" s="54" t="inlineStr">
+      <c r="C10" s="59" t="inlineStr">
         <is>
           <t>CA</t>
         </is>
       </c>
-      <c r="D10" s="54" t="inlineStr">
+      <c r="D10" s="59" t="inlineStr">
         <is>
           <t>NY</t>
         </is>
       </c>
-      <c r="E10" s="54" t="inlineStr">
+      <c r="E10" s="59" t="inlineStr">
         <is>
           <t>TX</t>
         </is>
@@ -3877,13 +4001,13 @@
           <t>State flat estimated tax rate</t>
         </is>
       </c>
-      <c r="C11" s="55" t="n">
+      <c r="C11" s="60" t="n">
         <v>0.06</v>
       </c>
-      <c r="D11" s="55" t="n">
+      <c r="D11" s="60" t="n">
         <v>0.05</v>
       </c>
-      <c r="E11" s="55" t="n">
+      <c r="E11" s="60" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3893,13 +4017,13 @@
           <t>Net SE income (annual)</t>
         </is>
       </c>
-      <c r="C12" s="56" t="n">
+      <c r="C12" s="33" t="n">
         <v>42600</v>
       </c>
-      <c r="D12" s="56" t="n">
+      <c r="D12" s="33" t="n">
         <v>60000</v>
       </c>
-      <c r="E12" s="56" t="n">
+      <c r="E12" s="33" t="n">
         <v>25000</v>
       </c>
     </row>
@@ -3909,13 +4033,13 @@
           <t>W-2 income</t>
         </is>
       </c>
-      <c r="C13" s="56" t="n">
-        <v>0</v>
-      </c>
-      <c r="D13" s="56" t="n">
+      <c r="C13" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="D13" s="33" t="n">
         <v>48000</v>
       </c>
-      <c r="E13" s="56" t="n">
+      <c r="E13" s="33" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3925,13 +4049,13 @@
           <t>Federal tax withheld from W-2</t>
         </is>
       </c>
-      <c r="C14" s="56" t="n">
-        <v>0</v>
-      </c>
-      <c r="D14" s="56" t="n">
+      <c r="C14" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="D14" s="33" t="n">
         <v>5400</v>
       </c>
-      <c r="E14" s="56" t="n">
+      <c r="E14" s="33" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3941,13 +4065,13 @@
           <t>Last year's total federal tax</t>
         </is>
       </c>
-      <c r="C15" s="56" t="n">
+      <c r="C15" s="33" t="n">
         <v>3200</v>
       </c>
-      <c r="D15" s="56" t="n">
+      <c r="D15" s="33" t="n">
         <v>8900</v>
       </c>
-      <c r="E15" s="56" t="n">
+      <c r="E15" s="33" t="n">
         <v>1800</v>
       </c>
     </row>
@@ -3957,13 +4081,13 @@
           <t>Last year's AGI</t>
         </is>
       </c>
-      <c r="C16" s="56" t="n">
+      <c r="C16" s="33" t="n">
         <v>38000</v>
       </c>
-      <c r="D16" s="56" t="n">
+      <c r="D16" s="33" t="n">
         <v>98000</v>
       </c>
-      <c r="E16" s="56" t="n">
+      <c r="E16" s="33" t="n">
         <v>24000</v>
       </c>
     </row>
@@ -3980,13 +4104,13 @@
           <t>Net SE income × 92.35% (SE base)</t>
         </is>
       </c>
-      <c r="C19" s="56" t="n">
+      <c r="C19" s="33" t="n">
         <v>39341</v>
       </c>
-      <c r="D19" s="56" t="n">
+      <c r="D19" s="33" t="n">
         <v>55410</v>
       </c>
-      <c r="E19" s="56" t="n">
+      <c r="E19" s="33" t="n">
         <v>23088</v>
       </c>
     </row>
@@ -3996,13 +4120,13 @@
           <t>Social Security (12.4%)</t>
         </is>
       </c>
-      <c r="C20" s="56" t="n">
+      <c r="C20" s="33" t="n">
         <v>4878</v>
       </c>
-      <c r="D20" s="56" t="n">
+      <c r="D20" s="33" t="n">
         <v>6871</v>
       </c>
-      <c r="E20" s="56" t="n">
+      <c r="E20" s="33" t="n">
         <v>2863</v>
       </c>
     </row>
@@ -4012,29 +4136,29 @@
           <t>Medicare (2.9%)</t>
         </is>
       </c>
-      <c r="C21" s="56" t="n">
+      <c r="C21" s="33" t="n">
         <v>1141</v>
       </c>
-      <c r="D21" s="56" t="n">
+      <c r="D21" s="33" t="n">
         <v>1607</v>
       </c>
-      <c r="E21" s="56" t="n">
+      <c r="E21" s="33" t="n">
         <v>669</v>
       </c>
     </row>
     <row r="22" ht="22" customHeight="1">
-      <c r="B22" s="57" t="inlineStr">
+      <c r="B22" s="61" t="inlineStr">
         <is>
           <t>Total SE tax</t>
         </is>
       </c>
-      <c r="C22" s="45" t="n">
+      <c r="C22" s="52" t="n">
         <v>6019</v>
       </c>
-      <c r="D22" s="45" t="n">
+      <c r="D22" s="52" t="n">
         <v>8478</v>
       </c>
-      <c r="E22" s="45" t="n">
+      <c r="E22" s="52" t="n">
         <v>3532</v>
       </c>
     </row>
@@ -4044,13 +4168,13 @@
           <t>AGI (W-2 + net SE − ½ SE tax)</t>
         </is>
       </c>
-      <c r="C23" s="56" t="n">
+      <c r="C23" s="33" t="n">
         <v>39591</v>
       </c>
-      <c r="D23" s="56" t="n">
+      <c r="D23" s="33" t="n">
         <v>103761</v>
       </c>
-      <c r="E23" s="56" t="n">
+      <c r="E23" s="33" t="n">
         <v>23234</v>
       </c>
     </row>
@@ -4060,13 +4184,13 @@
           <t>Standard deduction</t>
         </is>
       </c>
-      <c r="C24" s="56" t="n">
+      <c r="C24" s="33" t="n">
         <v>15750</v>
       </c>
-      <c r="D24" s="56" t="n">
+      <c r="D24" s="33" t="n">
         <v>31500</v>
       </c>
-      <c r="E24" s="56" t="n">
+      <c r="E24" s="33" t="n">
         <v>15750</v>
       </c>
     </row>
@@ -4076,45 +4200,45 @@
           <t>Taxable income</t>
         </is>
       </c>
-      <c r="C25" s="56" t="n">
+      <c r="C25" s="33" t="n">
         <v>23841</v>
       </c>
-      <c r="D25" s="56" t="n">
+      <c r="D25" s="33" t="n">
         <v>72261</v>
       </c>
-      <c r="E25" s="56" t="n">
+      <c r="E25" s="33" t="n">
         <v>7484</v>
       </c>
     </row>
     <row r="26" ht="22" customHeight="1">
-      <c r="B26" s="57" t="inlineStr">
+      <c r="B26" s="61" t="inlineStr">
         <is>
           <t>Federal income tax (bracket calc)</t>
         </is>
       </c>
-      <c r="C26" s="45" t="n">
+      <c r="C26" s="52" t="n">
         <v>2622</v>
       </c>
-      <c r="D26" s="45" t="n">
+      <c r="D26" s="52" t="n">
         <v>8195</v>
       </c>
-      <c r="E26" s="45" t="n">
+      <c r="E26" s="52" t="n">
         <v>748</v>
       </c>
     </row>
     <row r="27" ht="22" customHeight="1">
-      <c r="B27" s="57" t="inlineStr">
+      <c r="B27" s="61" t="inlineStr">
         <is>
           <t>State income tax</t>
         </is>
       </c>
-      <c r="C27" s="45" t="n">
+      <c r="C27" s="52" t="n">
         <v>1430</v>
       </c>
-      <c r="D27" s="45" t="n">
+      <c r="D27" s="52" t="n">
         <v>3613</v>
       </c>
-      <c r="E27" s="45" t="n">
+      <c r="E27" s="52" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4131,13 +4255,13 @@
           <t>Total federal owed (SE + income tax)</t>
         </is>
       </c>
-      <c r="C30" s="56" t="n">
+      <c r="C30" s="33" t="n">
         <v>8641</v>
       </c>
-      <c r="D30" s="56" t="n">
+      <c r="D30" s="33" t="n">
         <v>16673</v>
       </c>
-      <c r="E30" s="56" t="n">
+      <c r="E30" s="33" t="n">
         <v>4280</v>
       </c>
     </row>
@@ -4147,61 +4271,61 @@
           <t>Less: W-2 federal withholding</t>
         </is>
       </c>
-      <c r="C31" s="56" t="n">
-        <v>0</v>
-      </c>
-      <c r="D31" s="56" t="n">
+      <c r="C31" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="D31" s="33" t="n">
         <v>-5400</v>
       </c>
-      <c r="E31" s="56" t="n">
+      <c r="E31" s="33" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="32" ht="22" customHeight="1">
-      <c r="B32" s="57" t="inlineStr">
+      <c r="B32" s="61" t="inlineStr">
         <is>
           <t>Net federal owed (quarterly target ÷ 4)</t>
         </is>
       </c>
-      <c r="C32" s="45" t="n">
+      <c r="C32" s="52" t="n">
         <v>8641</v>
       </c>
-      <c r="D32" s="45" t="n">
+      <c r="D32" s="52" t="n">
         <v>11273</v>
       </c>
-      <c r="E32" s="45" t="n">
+      <c r="E32" s="52" t="n">
         <v>4280</v>
       </c>
     </row>
     <row r="33" ht="22" customHeight="1">
-      <c r="B33" s="57" t="inlineStr">
+      <c r="B33" s="61" t="inlineStr">
         <is>
           <t>Each federal quarterly payment</t>
         </is>
       </c>
-      <c r="C33" s="45" t="n">
+      <c r="C33" s="52" t="n">
         <v>2160</v>
       </c>
-      <c r="D33" s="45" t="n">
+      <c r="D33" s="52" t="n">
         <v>2818</v>
       </c>
-      <c r="E33" s="45" t="n">
+      <c r="E33" s="52" t="n">
         <v>1070</v>
       </c>
     </row>
     <row r="34" ht="22" customHeight="1">
-      <c r="B34" s="57" t="inlineStr">
+      <c r="B34" s="61" t="inlineStr">
         <is>
           <t>Each state quarterly payment</t>
         </is>
       </c>
-      <c r="C34" s="45" t="n">
+      <c r="C34" s="52" t="n">
         <v>358</v>
       </c>
-      <c r="D34" s="45" t="n">
+      <c r="D34" s="52" t="n">
         <v>903</v>
       </c>
-      <c r="E34" s="45" t="n">
+      <c r="E34" s="52" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4218,13 +4342,13 @@
           <t>100% of last year's tax (110% if AGI &gt; $150K)</t>
         </is>
       </c>
-      <c r="C37" s="56" t="n">
+      <c r="C37" s="33" t="n">
         <v>3200</v>
       </c>
-      <c r="D37" s="56" t="n">
+      <c r="D37" s="33" t="n">
         <v>8900</v>
       </c>
-      <c r="E37" s="56" t="n">
+      <c r="E37" s="33" t="n">
         <v>1800</v>
       </c>
     </row>
@@ -4234,44 +4358,44 @@
           <t>90% of this year's projected tax</t>
         </is>
       </c>
-      <c r="C38" s="56" t="n">
+      <c r="C38" s="33" t="n">
         <v>7777</v>
       </c>
-      <c r="D38" s="56" t="n">
+      <c r="D38" s="33" t="n">
         <v>15006</v>
       </c>
-      <c r="E38" s="56" t="n">
+      <c r="E38" s="33" t="n">
         <v>3852</v>
       </c>
     </row>
     <row r="39" ht="22" customHeight="1">
-      <c r="B39" s="57" t="inlineStr">
+      <c r="B39" s="61" t="inlineStr">
         <is>
           <t>Easier safe harbor — total to pay across 4 quarters</t>
         </is>
       </c>
-      <c r="C39" s="45" t="n">
+      <c r="C39" s="52" t="n">
         <v>3200</v>
       </c>
-      <c r="D39" s="45" t="n">
+      <c r="D39" s="52" t="n">
         <v>8900</v>
       </c>
-      <c r="E39" s="45" t="n">
+      <c r="E39" s="52" t="n">
         <v>1800</v>
       </c>
     </row>
     <row r="40" ht="22" customHeight="1">
-      <c r="B40" s="57">
+      <c r="B40" s="61">
         <f> safe-harbor quarterly amount</f>
         <v/>
       </c>
-      <c r="C40" s="45" t="n">
+      <c r="C40" s="52" t="n">
         <v>800</v>
       </c>
-      <c r="D40" s="45" t="n">
+      <c r="D40" s="52" t="n">
         <v>2225</v>
       </c>
-      <c r="E40" s="45" t="n">
+      <c r="E40" s="52" t="n">
         <v>450</v>
       </c>
     </row>
@@ -4311,7 +4435,7 @@
   </cols>
   <sheetData>
     <row r="2" ht="32" customHeight="1">
-      <c r="B2" s="34" t="inlineStr">
+      <c r="B2" s="42" t="inlineStr">
         <is>
           <t>IRS &amp; State Quarterly Tax Reference</t>
         </is>
@@ -4325,12 +4449,12 @@
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
-      <c r="B5" s="58" t="inlineStr">
+      <c r="B5" s="62" t="inlineStr">
         <is>
           <t>Q</t>
         </is>
       </c>
-      <c r="C5" s="44" t="inlineStr">
+      <c r="C5" s="51" t="inlineStr">
         <is>
           <t>Where do I actually pay federal quarterly tax?</t>
         </is>
@@ -4344,12 +4468,12 @@
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
-      <c r="B8" s="58" t="inlineStr">
+      <c r="B8" s="62" t="inlineStr">
         <is>
           <t>Q</t>
         </is>
       </c>
-      <c r="C8" s="44" t="inlineStr">
+      <c r="C8" s="51" t="inlineStr">
         <is>
           <t>Do I need to file Form 1040-ES?</t>
         </is>
@@ -4363,12 +4487,12 @@
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">
-      <c r="B11" s="58" t="inlineStr">
+      <c r="B11" s="62" t="inlineStr">
         <is>
           <t>Q</t>
         </is>
       </c>
-      <c r="C11" s="44" t="inlineStr">
+      <c r="C11" s="51" t="inlineStr">
         <is>
           <t>How does the state work?</t>
         </is>
@@ -4382,12 +4506,12 @@
       </c>
     </row>
     <row r="14" ht="22" customHeight="1">
-      <c r="B14" s="58" t="inlineStr">
+      <c r="B14" s="62" t="inlineStr">
         <is>
           <t>Q</t>
         </is>
       </c>
-      <c r="C14" s="44" t="inlineStr">
+      <c r="C14" s="51" t="inlineStr">
         <is>
           <t>What if my income is uneven across the year?</t>
         </is>
@@ -4401,12 +4525,12 @@
       </c>
     </row>
     <row r="17" ht="22" customHeight="1">
-      <c r="B17" s="58" t="inlineStr">
+      <c r="B17" s="62" t="inlineStr">
         <is>
           <t>Q</t>
         </is>
       </c>
-      <c r="C17" s="44" t="inlineStr">
+      <c r="C17" s="51" t="inlineStr">
         <is>
           <t>What's the actual penalty if I skip a quarter?</t>
         </is>
@@ -4420,12 +4544,12 @@
       </c>
     </row>
     <row r="20" ht="22" customHeight="1">
-      <c r="B20" s="58" t="inlineStr">
+      <c r="B20" s="62" t="inlineStr">
         <is>
           <t>Q</t>
         </is>
       </c>
-      <c r="C20" s="44" t="inlineStr">
+      <c r="C20" s="51" t="inlineStr">
         <is>
           <t>Can I overpay to be safe?</t>
         </is>
@@ -4439,12 +4563,12 @@
       </c>
     </row>
     <row r="23" ht="22" customHeight="1">
-      <c r="B23" s="58" t="inlineStr">
+      <c r="B23" s="62" t="inlineStr">
         <is>
           <t>Q</t>
         </is>
       </c>
-      <c r="C23" s="44" t="inlineStr">
+      <c r="C23" s="51" t="inlineStr">
         <is>
           <t>I had a huge year. Last year was tiny. Do I really only owe what last year's tax was × 4?</t>
         </is>
@@ -4458,12 +4582,12 @@
       </c>
     </row>
     <row r="26" ht="22" customHeight="1">
-      <c r="B26" s="58" t="inlineStr">
+      <c r="B26" s="62" t="inlineStr">
         <is>
           <t>Q</t>
         </is>
       </c>
-      <c r="C26" s="44" t="inlineStr">
+      <c r="C26" s="51" t="inlineStr">
         <is>
           <t>What if I miss a quarter and want to catch up?</t>
         </is>
@@ -4477,12 +4601,12 @@
       </c>
     </row>
     <row r="29" ht="22" customHeight="1">
-      <c r="B29" s="58" t="inlineStr">
+      <c r="B29" s="62" t="inlineStr">
         <is>
           <t>Q</t>
         </is>
       </c>
-      <c r="C29" s="44" t="inlineStr">
+      <c r="C29" s="51" t="inlineStr">
         <is>
           <t>Does this work if I'm both W-2 and self-employed?</t>
         </is>
@@ -4496,12 +4620,12 @@
       </c>
     </row>
     <row r="32" ht="22" customHeight="1">
-      <c r="B32" s="58" t="inlineStr">
+      <c r="B32" s="62" t="inlineStr">
         <is>
           <t>Q</t>
         </is>
       </c>
-      <c r="C32" s="44" t="inlineStr">
+      <c r="C32" s="51" t="inlineStr">
         <is>
           <t>Do I need to keep records of payments?</t>
         </is>

</xml_diff>